<commit_message>
Risiken ergaenzen: neues Blatt mit 10 Problemen und je 5 Gegenmassnahmen
- Neues Blatt 5 «Risiken»: Problem, warum es weh tut, fuenf konkrete
  Optionen dagegen, und wann es akut wird
- Saison-Spalte im Marktblatt: Golf laeuft April bis Oktober, Eishockey
  September bis April. Die beiden sind gegenlaeufig - zusammen ergibt das
  ein ganzjaehriges Geschaeft statt einer toten Wintersaison
- Beide Saisonfenster mit Quelle im Zahlenblatt belegt
- Blattnummern und Querverweise nachgezogen, Positionen auf Blatt 8
  werden jetzt berechnet statt fest verdrahtet

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TwwqEWQuBChyKpCZxs9c38
</commit_message>
<xml_diff>
--- a/coachgrid/Coach_Grid_Vereinsmodell.xlsx
+++ b/coachgrid/Coach_Grid_Vereinsmodell.xlsx
@@ -11,9 +11,10 @@
     <sheet name="2 Preise" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="3 Umsatz" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="4 Markt" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="5 Coach oder Verein" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="6 Fahrplan" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="7 Zahlen und Quellen" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="5 Risiken" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="6 Coach oder Verein" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="7 Fahrplan" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="8 Zahlen und Quellen" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -208,7 +209,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -295,6 +296,12 @@
     </xf>
     <xf numFmtId="164" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -1315,7 +1322,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Der Verein zahlt für Sichtbarkeit und erhält jede Anfrage in Kopie. Die Anfrage selbst geht an den Coach. So bleibt die Plattform eine Coach-Plattform (Blatt 5).</t>
+          <t>Der Verein zahlt für Sichtbarkeit und erhält jede Anfrage in Kopie. Die Anfrage selbst geht an den Coach. So bleibt die Plattform eine Coach-Plattform (Blatt 6).</t>
         </is>
       </c>
       <c r="C17" s="5" t="n"/>
@@ -1330,7 +1337,7 @@
       </c>
       <c r="B19" s="15" t="inlineStr">
         <is>
-          <t>Das Modell trägt — aber nur mit gestaffelten Preisen und mit Fokus auf grosse Vereine. Im realistischen Fall sind rund CHF 450'000 über drei Jahre erreichbar. Nächster Schritt: 50 Vereine aus der bestehenden Liste anschreiben und drei Pilotkunden gewinnen (Blatt 6).</t>
+          <t>Das Modell trägt — aber nur mit gestaffelten Preisen und mit Fokus auf grosse Vereine. Im realistischen Fall sind rund CHF 450'000 über drei Jahre erreichbar. Nächster Schritt: 50 Vereine aus der bestehenden Liste anschreiben und drei Pilotkunden gewinnen (Blatt 7).</t>
         </is>
       </c>
       <c r="C19" s="5" t="n"/>
@@ -2302,15 +2309,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -2345,21 +2353,26 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
+          <t>Saison</t>
+        </is>
+      </c>
+      <c r="E4" s="7" t="inlineStr">
+        <is>
           <t>Stufe</t>
         </is>
       </c>
-      <c r="E4" s="7" t="inlineStr">
+      <c r="F4" s="7" t="inlineStr">
         <is>
           <t>Umsatz bei 100 %</t>
         </is>
       </c>
-      <c r="F4" s="7" t="inlineStr">
+      <c r="G4" s="7" t="inlineStr">
         <is>
           <t>Warum in dieser Reihenfolge</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="40" customHeight="1">
+    <row r="5" ht="46" customHeight="1">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Golf</t>
@@ -2371,22 +2384,27 @@
       <c r="C5" s="31" t="n">
         <v>100</v>
       </c>
-      <c r="D5" s="19" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>April bis Oktober</t>
+        </is>
+      </c>
+      <c r="E5" s="19" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="E5" s="20">
+      <c r="F5" s="20">
         <f>B5*'2 Preise'!C8</f>
         <v/>
       </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>Höchste Zahlungskraft: eigener Platz, Geschäftsführung, Marketingbudget.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="40" customHeight="1">
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Höchste Zahlungskraft: eigener Platz, Geschäftsführung, Marketingbudget. Im Winter ruht der Betrieb.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="46" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>Tennis</t>
@@ -2398,22 +2416,27 @@
       <c r="C6" s="31" t="n">
         <v>900</v>
       </c>
-      <c r="D6" s="19" t="inlineStr">
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Aussenplätze April bis Oktober, Halle ganzjährig</t>
+        </is>
+      </c>
+      <c r="E6" s="19" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E6" s="20">
+      <c r="F6" s="20">
         <f>B6*'2 Preise'!C9</f>
         <v/>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>Grösste Zahl an Clubs mit eigener Anlage und eigenen Trainern.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="40" customHeight="1">
+    <row r="7" ht="46" customHeight="1">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Schwimmen</t>
@@ -2425,22 +2448,27 @@
       <c r="C7" s="31" t="n">
         <v>175</v>
       </c>
-      <c r="D7" s="19" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>ganzjährig (Hallenbad)</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E7" s="20">
+      <c r="F7" s="20">
         <f>B7*'2 Preise'!C9</f>
         <v/>
       </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>Laufendes Kursgeschäft; dort wird ohnehin nach Angeboten gesucht.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="40" customHeight="1">
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Laufendes Kursgeschäft ohne Saisonlücke; dort wird ohnehin nach Angeboten gesucht.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="46" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Reiten und Eishockey</t>
@@ -2452,18 +2480,23 @@
       <c r="C8" s="31" t="n">
         <v>450</v>
       </c>
-      <c r="D8" s="19" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Eishockey September bis April, Reiten ganzjährig</t>
+        </is>
+      </c>
+      <c r="E8" s="19" t="inlineStr">
         <is>
           <t>M</t>
         </is>
       </c>
-      <c r="E8" s="20">
+      <c r="F8" s="20">
         <f>B8*'2 Preise'!C9</f>
         <v/>
       </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>Grosser Nachwuchsstab, Reitbetriebe entscheiden schnell.</t>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>Eishockey füllt genau die Monate, in denen Golf stillsteht.</t>
         </is>
       </c>
     </row>
@@ -2482,11 +2515,12 @@
         <v/>
       </c>
       <c r="D9" s="28" t="inlineStr"/>
-      <c r="E9" s="32">
-        <f>SUM(E5:E8)</f>
-        <v/>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="E9" s="28" t="inlineStr"/>
+      <c r="F9" s="32">
+        <f>SUM(F5:F8)</f>
+        <v/>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>Obergrenze, wenn jeder Verein der Liste zahlt. Keine Planzahl.</t>
         </is>
@@ -2500,17 +2534,18 @@
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>414 Vereine sind mit Name, Telefon und Mailadresse direkt ansprechbar. Golf und die grossen Tennisclubs zuerst: dort sind Budget, feste Ansprechpartner und eigene Trainer vorhanden. Schwimmvereine folgen, weil dort das Kursgeschäft läuft.</t>
+          <t>414 Vereine sind mit Name, Telefon und Mailadresse direkt ansprechbar. Golf zuerst, weil dort Budget und feste Ansprechpartner vorhanden sind — aber Golf steht von November bis März still. Eishockey läuft genau dann. Wer beide Sportarten im Kundenstamm hat, hat ganzjährig Anfragen statt einer toten Wintersaison. Risiken und Gegenmassnahmen auf Blatt 5.</t>
         </is>
       </c>
       <c r="C11" s="5" t="n"/>
       <c r="D11" s="5" t="n"/>
       <c r="E11" s="5" t="n"/>
-      <c r="F11" s="6" t="n"/>
+      <c r="F11" s="5" t="n"/>
+      <c r="G11" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B11:G11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -2518,6 +2553,339 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="62" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Was schiefgehen kann</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Zehn Probleme, die im Vereinsgeschäft auftreten — und was dagegen hilft.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>Problem</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Warum es weh tut</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>Was man dagegen tun kann</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>Wann es akut wird</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="104" customHeight="1">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>Golf ist ein Saisongeschäft</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Die Plätze sind etwa von April bis Oktober offen, in den Bergen kürzer. Von November bis März kommen kaum Anfragen — der Club sieht keinen Gegenwert und stellt das Abo infrage.</t>
+        </is>
+      </c>
+      <c r="C5" s="33" t="inlineStr">
+        <is>
+          <t>1. Jahresvertrag statt Monatsabo: der Nutzen wird über die Saison gemessen, nicht über den Monat.
+2. Eishockey als Gegengewicht aufnehmen — dessen Saison läuft September bis April.
+3. Die Wintermonate im Vertrag als Vorbereitungszeit ausweisen: Profile, Fotos, Kursangebote für die neue Saison.
+4. Reporting pro Saison statt pro Monat verschicken.
+5. Im Winter verkaufen, im Frühling starten — dann fallen Budgetbeschluss und Saisonstart zusammen.</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>ab dem ersten Winter</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="104" customHeight="1">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Vereine entscheiden langsam</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Der Vorstand arbeitet ehrenamtlich und tagt oft nur quartalsweise. Grössere Ausgaben brauchen die Generalversammlung. Aus einem Gespräch werden schnell sechs Monate bis zur Unterschrift.</t>
+        </is>
+      </c>
+      <c r="C6" s="33" t="inlineStr">
+        <is>
+          <t>1. Direkt beim Geschäftsführer oder Sekretariat ansetzen statt beim Gesamtvorstand.
+2. Den Preis so wählen, dass er unter der Genehmigungsschwelle des Vorstands liegt.
+3. Eine kostenlose Testphase bis zur nächsten Generalversammlung anbieten.
+4. Vertragsbeginn auf den Start des Vereinsjahrs legen.
+5. Den Verkauf ins Budgetfenster im Herbst legen, nicht ins Frühjahr.</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>sofort, im ersten Gespräch</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="104" customHeight="1">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Den meisten Vereinen fehlt schlicht das Geld</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>82 Prozent der Schweizer Sportvereine haben keine bezahlte Person, die durchschnittlichen Jahreseinnahmen liegen bei CHF 69'000. Ein Abo über CHF 10'000 wäre dort ein Siebtel des Budgets.</t>
+        </is>
+      </c>
+      <c r="C7" s="33" t="inlineStr">
+        <is>
+          <t>1. Nur Vereine mit eigener Anlage ansprechen — dort gibt es Fixkosten und damit eine Buchhaltung.
+2. Kleinere Vereine gar nicht als Verein verkaufen, sondern deren Coaches einzeln zu CHF 399.
+3. Zahlung aus dem Sponsoring- oder Marketingtopf statt aus der Vereinskasse vorschlagen.
+4. Abrechnung pro Coach statt Pauschale, damit der Betrag mitwächst.
+5. Rahmenvertrag über einen Verband prüfen statt Einzelverträge.</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>bei jedem zweiten Kontakt</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="104" customHeight="1">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Coaches fühlen sich übergangen</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Wenn der Verein den Zugang bezahlt, entsteht schnell der Eindruck, das Profil gehöre dem Verein. Genau die Coaches, wegen denen die Plattform existiert, verlieren dann das Interesse.</t>
+        </is>
+      </c>
+      <c r="C8" s="33" t="inlineStr">
+        <is>
+          <t>1. Die Anfrage geht an den Coach, der Verein bekommt sie in Kopie (Blatt 6).
+2. Das Profil bleibt beim Coach, auch wenn er den Verein verlässt.
+3. Bewertungen und Referenzen gehören dem Coach, nicht dem Vereinskonto.
+4. Coaches vor der Unterschrift des Vereins informieren, nicht danach.
+5. Den Vereinsnamen als Zusatz im Profil führen, nicht als Absender.</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>sobald der erste Verein aktiv ist</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="104" customHeight="1">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>Der Coach arbeitet privat weiter</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>Der Verein zahlt, die Anfragen laufen aber an ihm vorbei in private Stunden. Dann bezahlt der Verein die Sichtbarkeit für ein Geschäft, an dem er nichts verdient.</t>
+        </is>
+      </c>
+      <c r="C9" s="33" t="inlineStr">
+        <is>
+          <t>1. Preisuntergrenze im Vertrag: Privatstunden eines Vereinscoaches liegen mindestens auf Vereinsniveau.
+2. Ein zweites, privates Profil nur mit schriftlicher Freigabe des Vereins.
+3. Der Zugangscode erlischt beim Vereinsaustritt.
+4. Das Dashboard zeigt dem Verein alle Anfragen an seine Coaches.
+5. Verstoss führt zum Entzug des Zugangs, nicht zu einer Diskussion.</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>nach den ersten Monaten</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="104" customHeight="1">
+      <c r="A10" s="13" t="inlineStr">
+        <is>
+          <t>Zu wenig Rücklauf, keine Verlängerung</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>Wir können keine neuen Mitglieder garantieren. Bleiben die Anfragen aus, verlängert der Verein nach einem Jahr nicht — und erzählt es den Nachbarvereinen.</t>
+        </is>
+      </c>
+      <c r="C10" s="33" t="inlineStr">
+        <is>
+          <t>1. Erfolgskriterien vor der Unterschrift schriftlich festhalten.
+2. Monatliches Reporting ab dem ersten Tag, auch wenn die Zahlen klein sind.
+3. Erstes Jahr zum halben Preis gegen das Recht, den Verein als Referenz zu nennen.
+4. Ausstiegsmöglichkeit nach zwölf Monaten statt Streit um die Restlaufzeit.
+5. Bei schwachen Zahlen nachbessern (mehr Sichtbarkeit) statt Geld zurückzahlen.</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>nach zwölf Monaten</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="104" customHeight="1">
+      <c r="A11" s="13" t="inlineStr">
+        <is>
+          <t>Wenige Kunden tragen den ganzen Umsatz</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Zwanzig grosse Vereine bringen den Umsatz von zweihundert kleinen — kündigen drei davon, bricht ein Sechstel des Geschäfts weg.</t>
+        </is>
+      </c>
+      <c r="C11" s="33" t="inlineStr">
+        <is>
+          <t>1. Kein Verein darf mehr als 15 Prozent des Vereinsumsatzes ausmachen.
+2. Das Einzelcoach-Geschäft bewusst weiterführen, nicht ersetzen.
+3. Vertragsenden über das Jahr verteilen statt alle per 31. Dezember.
+4. Nutzung des Dashboards als Frühwarnsignal beobachten.
+5. Mindestens zwei Sportarten im Kundenstamm halten.</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>ab dem zehnten Kunden</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="104" customHeight="1">
+      <c r="A12" s="13" t="inlineStr">
+        <is>
+          <t>Onboarding von 40 Coaches kostet Zeit</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Ein Grossverein bedeutet vierzig Profile mit Foto, Text und Qualifikationen. Ohne Prozess verbrennt das mehr Zeit, als das Abo einbringt.</t>
+        </is>
+      </c>
+      <c r="C12" s="33" t="inlineStr">
+        <is>
+          <t>1. Selbstregistrierung der Coaches über einen Vereinscode.
+2. Einmalige Einrichtungsgebühr, die den Aufwand deckt.
+3. Ein Ansprechpartner im Verein, der die Coaches sammelt und nachfasst.
+4. Profile per Liste importieren statt einzeln erfassen.
+5. Den Zeitaufwand im Pilot messen und in den Preis der nächsten Stufe einrechnen.</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>beim ersten Grossverein</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="104" customHeight="1">
+      <c r="A13" s="13" t="inlineStr">
+        <is>
+          <t>Der Verband baut es selbst</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Swiss Tennis, Swiss Golf oder Swiss Aquatics haben die Vereine bereits als Mitglieder. Bauen sie ein eigenes Verzeichnis, verlieren wir den Zugang zu genau dieser Gruppe.</t>
+        </is>
+      </c>
+      <c r="C13" s="33" t="inlineStr">
+        <is>
+          <t>1. Den Verband als Partner ansprechen, bevor er es selbst versucht.
+2. Auf Buchung und Lektion setzen — eine reine Auflistung kann jeder Verband selbst.
+3. Die ersten Clubs mit einer Exklusivität in ihrer Region binden.
+4. Schnell sein: ein Verbandsprojekt braucht Jahre, wir brauchen Monate.
+5. Die Marke bei den Coaches aufbauen — die bleiben, auch wenn der Verein wechselt.</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>im zweiten Jahr</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="104" customHeight="1">
+      <c r="A14" s="13" t="inlineStr">
+        <is>
+          <t>Kaltakquise per Mail</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Wir schreiben Vereine an, die uns nicht kennen. Ohne Sorgfalt landet das im Spam und schadet der Absenderadresse für alle künftigen Mails.</t>
+        </is>
+      </c>
+      <c r="C14" s="33" t="inlineStr">
+        <is>
+          <t>1. Nur allgemeine Vereinsadressen verwenden, keine privaten Adressen von Vorstandsmitgliedern.
+2. Abmeldemöglichkeit in jeder Mail, Absender und Kontakt klar erkennbar.
+3. Nach einem Widerspruch die Adresse dauerhaft aus der Liste nehmen.
+4. Höchstens zweimal schreiben, danach telefonisch nachfassen.
+5. In Wellen von 50 Adressen versenden statt 414 auf einmal.</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>ab der ersten Welle</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="58" customHeight="1">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>FAZIT</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>Kein Problem auf dieser Liste kippt das Modell — aber vier davon treffen schon im ersten Jahr: die Winterlücke bei Golf, die langsamen Vereinsentscheide, das fehlende Budget bei kleinen Vereinen und die Sorge der Coaches. Alle vier lassen sich mit Vertragsgestaltung und der Wahl der Zielgruppe entschärfen, nicht mit Entwicklung. Genau das ist im Fahrplan auf Blatt 7 abgebildet.</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="6" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B16:D16"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2764,7 +3132,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2915,7 +3283,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Termine wahrnehmen, Blatt 2 und 5 als Gesprächsgrundlage nutzen.</t>
+          <t>Termine wahrnehmen, Blatt 2 und 6 als Gesprächsgrundlage nutzen.</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -3076,13 +3444,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -3145,7 +3513,7 @@
           <t>18'310</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3167,7 +3535,7 @@
           <t>2'200'000</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3189,7 +3557,7 @@
           <t>CHF 69'000</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3211,7 +3579,7 @@
           <t>82 %</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3233,7 +3601,7 @@
           <t>41 %</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3255,7 +3623,7 @@
           <t>rund 900</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3277,7 +3645,7 @@
           <t>über 90</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3299,7 +3667,7 @@
           <t>175</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3321,7 +3689,7 @@
           <t>1'345</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3343,7 +3711,7 @@
           <t>22 %</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3365,7 +3733,7 @@
           <t>67 %</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3379,274 +3747,346 @@
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
+          <t>Saison National League Eishockey</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>September bis April</t>
+        </is>
+      </c>
+      <c r="C17" s="34" t="inlineStr">
+        <is>
+          <t>belegt</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>Spielplan National League: Qualifikation September bis März, Playoffs bis April</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Saison Golfplätze Schweiz</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>April bis Oktober</t>
+        </is>
+      </c>
+      <c r="C18" s="34" t="inlineStr">
+        <is>
+          <t>belegt</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Saisonzeiten der Golfplätze, Graubünden Ferien. Je nach Höhenlage kürzer</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
           <t>Kontaktierbare Vereine in unserer Liste</t>
         </is>
       </c>
-      <c r="B17" s="13" t="inlineStr">
+      <c r="B19" s="13" t="inlineStr">
         <is>
           <t>414</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C19" s="34" t="inlineStr">
         <is>
           <t>eigene Erhebung</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>Eigene Liste vom 28.07.2026: Golf 103, Tennis 99, Schwimmen 180, Reiten und Eishockey 32</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Eingaben, die im Pilot gemessen werden</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="30" customHeight="1">
-      <c r="A20" s="7" t="inlineStr">
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>Eingabe</t>
         </is>
       </c>
-      <c r="B20" s="7" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Im Modell</t>
         </is>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>Art</t>
         </is>
       </c>
-      <c r="D20" s="7" t="inlineStr">
+      <c r="D22" s="7" t="inlineStr">
         <is>
           <t>Wird gemessen durch</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Preis pro Coach und Jahr</t>
-        </is>
-      </c>
-      <c r="B21" s="13" t="inlineStr">
-        <is>
-          <t>CHF 399</t>
-        </is>
-      </c>
-      <c r="C21" s="33" t="inlineStr">
-        <is>
-          <t>Eingabe</t>
-        </is>
-      </c>
-      <c r="D21" s="4" t="inlineStr">
-        <is>
-          <t>Bereits im Einsatz, auf Blatt 2 änderbar</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="24" customHeight="1">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>Antwortquote auf ein Anschreiben</t>
-        </is>
-      </c>
-      <c r="B22" s="13" t="inlineStr">
-        <is>
-          <t>12 / 20 / 30 %</t>
-        </is>
-      </c>
-      <c r="C22" s="33" t="inlineStr">
-        <is>
-          <t>Eingabe</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>Erste Welle an 50 Vereine, Woche 3–4</t>
         </is>
       </c>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Anteil, der Kunde wird</t>
+          <t>Preis pro Coach und Jahr</t>
         </is>
       </c>
       <c r="B23" s="13" t="inlineStr">
         <is>
-          <t>8 / 15 / 25 %</t>
-        </is>
-      </c>
-      <c r="C23" s="33" t="inlineStr">
+          <t>CHF 399</t>
+        </is>
+      </c>
+      <c r="C23" s="35" t="inlineStr">
         <is>
           <t>Eingabe</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Gespräche in Woche 5–8</t>
+          <t>Bereits im Einsatz, auf Blatt 2 änderbar</t>
         </is>
       </c>
     </row>
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Verlängerung im Folgejahr</t>
+          <t>Antwortquote auf ein Anschreiben</t>
         </is>
       </c>
       <c r="B24" s="13" t="inlineStr">
         <is>
-          <t>75 / 85 / 90 %</t>
-        </is>
-      </c>
-      <c r="C24" s="33" t="inlineStr">
+          <t>12 / 20 / 30 %</t>
+        </is>
+      </c>
+      <c r="C24" s="35" t="inlineStr">
         <is>
           <t>Eingabe</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Erst nach zwölf Monaten messbar</t>
+          <t>Erste Welle an 50 Vereine, Woche 3–4</t>
         </is>
       </c>
     </row>
     <row r="25" ht="24" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
+          <t>Anteil, der Kunde wird</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>8 / 15 / 25 %</t>
+        </is>
+      </c>
+      <c r="C25" s="35" t="inlineStr">
+        <is>
+          <t>Eingabe</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Gespräche in Woche 5–8</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>Verlängerung im Folgejahr</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="inlineStr">
+        <is>
+          <t>75 / 85 / 90 %</t>
+        </is>
+      </c>
+      <c r="C26" s="35" t="inlineStr">
+        <is>
+          <t>Eingabe</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>Erst nach zwölf Monaten messbar</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
           <t>Coaches pro Verein</t>
         </is>
       </c>
-      <c r="B25" s="13" t="inlineStr">
+      <c r="B27" s="13" t="inlineStr">
         <is>
           <t>10 bis 40</t>
         </is>
       </c>
-      <c r="C25" s="33" t="inlineStr">
+      <c r="C27" s="35" t="inlineStr">
         <is>
           <t>Eingabe</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>Wird im Erstgespräch erfasst</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
         <is>
           <t>Quellen</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="34" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="36" t="inlineStr">
         <is>
           <t>Vereinsstudie 2022, Swiss Olympic</t>
         </is>
       </c>
-      <c r="B28" s="35" t="inlineStr">
+      <c r="B30" s="37" t="inlineStr">
         <is>
           <t>https://www.swissolympic.ch/dam/jcr:e13bfb8d-92a6-41a3-89e4-b80d30c2d23c/Vereinsstudie%202022_DE_Web.pdf</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="34" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="36" t="inlineStr">
         <is>
           <t>Observatorium Sport und Bewegung Schweiz</t>
         </is>
       </c>
-      <c r="B29" s="35" t="inlineStr">
+      <c r="B31" s="37" t="inlineStr">
         <is>
           <t>https://www.sportobs.ch/inhalte/Indikatoren_PDF_neu/Ind_22_Sportobs.pdf</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="34" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="36" t="inlineStr">
         <is>
           <t>Sport Schweiz 2020, BASPO</t>
         </is>
       </c>
-      <c r="B30" s="35" t="inlineStr">
+      <c r="B32" s="37" t="inlineStr">
         <is>
           <t>https://www.sportobs.ch/inhalte/Downloads/Bro_Sport_Schweiz_2020_d_WEB.pdf</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="A31" s="34" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="36" t="inlineStr">
         <is>
           <t>Swiss Aquatics, Mitgliedvereine</t>
         </is>
       </c>
-      <c r="B31" s="35" t="inlineStr">
+      <c r="B33" s="37" t="inlineStr">
         <is>
           <t>https://www.swiss-aquatics.ch/verband/mitglieder/alle-mitgliedvereine/</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="34" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="36" t="inlineStr">
         <is>
           <t>Swiss Tennis</t>
         </is>
       </c>
-      <c r="B32" s="35" t="inlineStr">
+      <c r="B34" s="37" t="inlineStr">
         <is>
           <t>https://www.swisstennis.ch/de/</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="34" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="36" t="inlineStr">
         <is>
           <t>Swiss Golf</t>
         </is>
       </c>
-      <c r="B33" s="35" t="inlineStr">
+      <c r="B35" s="37" t="inlineStr">
         <is>
           <t>https://www.swissgolf.ch/</t>
         </is>
       </c>
     </row>
-    <row r="35" ht="58" customHeight="1">
-      <c r="A35" s="14" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="36" t="inlineStr">
+        <is>
+          <t>Saisonzeiten Golfplätze, Graubünden Ferien</t>
+        </is>
+      </c>
+      <c r="B36" s="37" t="inlineStr">
+        <is>
+          <t>https://www.graubuenden.ch/de/news/saisonzeiten-golfplaetze</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="36" t="inlineStr">
+        <is>
+          <t>Spielplan National League</t>
+        </is>
+      </c>
+      <c r="B37" s="37" t="inlineStr">
+        <is>
+          <t>https://www.sihf.ch/</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="58" customHeight="1">
+      <c r="A39" s="14" t="inlineStr">
         <is>
           <t>FAZIT</t>
         </is>
       </c>
-      <c r="B35" s="15" t="inlineStr">
-        <is>
-          <t>Elf Marktzahlen sind belegt und verlinkt, eine stammt aus der eigenen Erhebung. Fünf Werte sind Eingaben — sie treiben das Ergebnis und werden im 90-Tage-Pilot durch gemessene Zahlen ersetzt. Bis dahin ist jedes Umsatzszenario eine Rechnung, keine Prognose.</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="n"/>
-      <c r="D35" s="6" t="n"/>
+      <c r="B39" s="15" t="inlineStr">
+        <is>
+          <t>Dreizehn Marktzahlen sind belegt und verlinkt, eine stammt aus der eigenen Erhebung. Fünf Werte sind Eingaben — sie treiben das Ergebnis und werden im 90-Tage-Pilot durch gemessene Zahlen ersetzt. Bis dahin ist jedes Umsatzszenario eine Rechnung, keine Prognose.</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="n"/>
+      <c r="D39" s="6" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
     <mergeCell ref="B33:D33"/>
-    <mergeCell ref="B28:D28"/>
+    <mergeCell ref="B36:D36"/>
+    <mergeCell ref="B37:D37"/>
     <mergeCell ref="B31:D31"/>
     <mergeCell ref="B32:D32"/>
     <mergeCell ref="B35:D35"/>
     <mergeCell ref="B30:D30"/>
-    <mergeCell ref="B29:D29"/>
+    <mergeCell ref="B39:D39"/>
+    <mergeCell ref="B34:D34"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Vereinspreise: Aufschlag statt Rabatt gegenüber Einzelcoach
Vereine zahlen neu CHF 420–549 pro Coach/Jahr (immer über dem
Einzelpreis von CHF 399), weil sie Club-Dashboard, zentrale
Abrechnung und Vereinsprofil erhalten.

- Blatt 2: Tiers S/M/L/XL zeigen Preis pro Coach (blau) + Aufschlag in %
- Vergleichstabelle zeigt Mehrkosten Vereinspaket vs. Einzelanmeldungen
- Blatt 4: «Umsatz bei 100 %» referenziert Jahresbeispiel-Spalte (E)
- Blatt 3: Optimistisch-Input von CHF 6'900 auf CHF 9'000 angehoben
- Blatt 1: Erkenntnis #1 erklärt Premium-Logik statt Rabatt-Logik

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TwwqEWQuBChyKpCZxs9c38
</commit_message>
<xml_diff>
--- a/coachgrid/Coach_Grid_Vereinsmodell.xlsx
+++ b/coachgrid/Coach_Grid_Vereinsmodell.xlsx
@@ -130,12 +130,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F7D4CF"/>
+        <fgColor rgb="00FBE7C0"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FBE7C0"/>
+        <fgColor rgb="00F7D4CF"/>
       </patternFill>
     </fill>
   </fills>
@@ -209,7 +209,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -258,10 +258,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -270,16 +273,7 @@
     <xf numFmtId="3" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -300,10 +294,13 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -396,7 +393,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Einheitspreis gegen Summe der Einzelanmeldungen</a:t>
+              <a:t>Vereinspreis vs. Einzelanmeldungen (CHF / Jahr)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -411,30 +408,6 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'2 Preise'!B15</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln>
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'2 Preise'!$A$16:$A$23</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'2 Preise'!$B$16:$B$23</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
               <f>'2 Preise'!C15</f>
             </strRef>
           </tx>
@@ -445,12 +418,36 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'2 Preise'!$A$16:$A$23</f>
+              <f>'2 Preise'!$A$16:$A$22</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'2 Preise'!$C$16:$C$23</f>
+              <f>'2 Preise'!$C$16:$C$22</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'2 Preise'!D15</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'2 Preise'!$A$16:$A$22</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'2 Preise'!$D$16:$D$22</f>
             </numRef>
           </val>
         </ser>
@@ -473,7 +470,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Coaches im Verein</a:t>
+                  <a:t>Anzahl Coaches im Verein</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -1287,12 +1284,12 @@
     <row r="15" ht="52" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>Ein Preis für alle geht nicht</t>
+          <t>Vereine zahlen mehr als einzelne Coaches</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>CHF 10'000 im Jahr entsprechen 25 Coaches zum Einzelpreis. Ein Verein mit 15 Coaches zahlt damit mehr, als wenn sich seine Coaches einzeln anmelden. Lösung: Staffelpreise (Blatt 2).</t>
+          <t>Ein einzelner Coach bezahlt CHF 399 pro Jahr. Vereine zahlen pro Coach CHF 420 bis CHF 549, weil sie zusätzlich Club-Dashboard, zentrale Abrechnung und ein Vereinsprofil erhalten. Das ist kein Rabatt, sondern ein Aufschlag für mehr Leistung (Blatt 2).</t>
         </is>
       </c>
       <c r="C15" s="5" t="n"/>
@@ -1383,14 +1380,14 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Der Vereinspreis muss unter der Summe der Einzelanmeldungen liegen.</t>
+          <t>Einzelcoach CHF 399 / Jahr. Vereine zahlen pro Coach einen Aufschlag — dafür erhalten sie Club-Dashboard, zentrale Abrechnung und Vereinsprofil.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>Preis pro Coach und Jahr (heute)</t>
+          <t>Einzelcoach — Preis pro Jahr (heute)</t>
         </is>
       </c>
       <c r="B4" s="16" t="n">
@@ -1405,7 +1402,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>Staffelpreise</t>
+          <t>Vereinspakete — Preis pro Coach und Jahr</t>
         </is>
       </c>
     </row>
@@ -1422,22 +1419,22 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>Preis pro Jahr</t>
+          <t>Pro Coach / Jahr</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Preis pro Monat</t>
+          <t>Monatlich</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>Ersparnis pro Jahr</t>
+          <t>Jahresbeispiel</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Preis pro Coach</t>
+          <t>Aufschlag vs. Einzelcoach</t>
         </is>
       </c>
     </row>
@@ -1449,21 +1446,22 @@
       </c>
       <c r="B8" s="19" t="inlineStr">
         <is>
-          <t>1 – 10</t>
+          <t>1 – 5</t>
         </is>
       </c>
       <c r="C8" s="16" t="n">
-        <v>2490</v>
-      </c>
-      <c r="D8" s="16" t="n">
-        <v>249</v>
-      </c>
-      <c r="E8" s="20">
-        <f>D8*12-C8</f>
-        <v/>
-      </c>
-      <c r="F8" s="21">
-        <f>C8/10</f>
+        <v>549</v>
+      </c>
+      <c r="D8" s="20">
+        <f>C8/12</f>
+        <v/>
+      </c>
+      <c r="E8" s="21">
+        <f>C8*4</f>
+        <v/>
+      </c>
+      <c r="F8" s="22">
+        <f>(C8-$B$4)/$B$4</f>
         <v/>
       </c>
     </row>
@@ -1475,21 +1473,22 @@
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>11 – 25</t>
+          <t>6 – 15</t>
         </is>
       </c>
       <c r="C9" s="16" t="n">
-        <v>4900</v>
-      </c>
-      <c r="D9" s="16" t="n">
         <v>490</v>
       </c>
-      <c r="E9" s="20">
-        <f>D9*12-C9</f>
-        <v/>
-      </c>
-      <c r="F9" s="21">
-        <f>C9/18</f>
+      <c r="D9" s="20">
+        <f>C9/12</f>
+        <v/>
+      </c>
+      <c r="E9" s="21">
+        <f>C9*10</f>
+        <v/>
+      </c>
+      <c r="F9" s="22">
+        <f>(C9-$B$4)/$B$4</f>
         <v/>
       </c>
     </row>
@@ -1501,21 +1500,22 @@
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>26 – 40</t>
+          <t>16 – 30</t>
         </is>
       </c>
       <c r="C10" s="16" t="n">
-        <v>9900</v>
-      </c>
-      <c r="D10" s="16" t="n">
-        <v>990</v>
-      </c>
-      <c r="E10" s="20">
-        <f>D10*12-C10</f>
-        <v/>
-      </c>
-      <c r="F10" s="21">
-        <f>C10/33</f>
+        <v>449</v>
+      </c>
+      <c r="D10" s="20">
+        <f>C10/12</f>
+        <v/>
+      </c>
+      <c r="E10" s="21">
+        <f>C10*20</f>
+        <v/>
+      </c>
+      <c r="F10" s="22">
+        <f>(C10-$B$4)/$B$4</f>
         <v/>
       </c>
     </row>
@@ -1527,28 +1527,29 @@
       </c>
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>ab 41</t>
+          <t>ab 31</t>
         </is>
       </c>
       <c r="C11" s="16" t="n">
-        <v>14900</v>
-      </c>
-      <c r="D11" s="16" t="n">
-        <v>1490</v>
-      </c>
-      <c r="E11" s="20">
-        <f>D11*12-C11</f>
-        <v/>
-      </c>
-      <c r="F11" s="21">
-        <f>C11/50</f>
-        <v/>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="22" t="inlineStr">
-        <is>
-          <t>Wer jährlich zahlt, spart sichtbar. Beim grossen Verein sind das CHF 1'980.</t>
+        <v>420</v>
+      </c>
+      <c r="D11" s="20">
+        <f>C11/12</f>
+        <v/>
+      </c>
+      <c r="E11" s="21">
+        <f>C11*35</f>
+        <v/>
+      </c>
+      <c r="F11" s="22">
+        <f>(C11-$B$4)/$B$4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="28" customHeight="1">
+      <c r="A12" s="23" t="inlineStr">
+        <is>
+          <t>Jahresbeispiel: S = 4 Coaches, M = 10, L = 20, XL = 35. Inklusive: Club-Dashboard, Sammelrechnung, Analytics, Vereinsprofil auf thecoachgrid.com.</t>
         </is>
       </c>
       <c r="B12" s="5" t="n"/>
@@ -1560,240 +1561,222 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Gegenprobe: ein Einheitspreis von CHF 10'000</t>
+          <t>Jahreskosten im Vergleich: Vereinspaket vs. Einzelanmeldungen</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Coaches im Verein</t>
+          <t>Coaches</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Einzeln angemeldet</t>
+          <t>Stufe</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Einheitspreis</t>
+          <t>Vereinspreis total</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Differenz</t>
+          <t>Einzeln total</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Verhältnis</t>
+          <t>Mehrkosten</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Ergebnis</t>
+          <t>Aufschlag</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="23" t="n">
+      <c r="A16" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C16" s="20">
+        <f>3*$C$8</f>
+        <v/>
+      </c>
+      <c r="D16" s="20">
+        <f>3*$B$4</f>
+        <v/>
+      </c>
+      <c r="E16" s="25">
+        <f>C16-D16</f>
+        <v/>
+      </c>
+      <c r="F16" s="22">
+        <f>(C16-D16)/D16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="B16" s="21">
-        <f>A16*$B$4</f>
-        <v/>
-      </c>
-      <c r="C16" s="21" t="n">
-        <v>10000</v>
-      </c>
-      <c r="D16" s="21">
-        <f>C16-B16</f>
-        <v/>
-      </c>
-      <c r="E16" s="24">
-        <f>C16/B16</f>
-        <v/>
-      </c>
-      <c r="F16" s="25" t="inlineStr">
-        <is>
-          <t>Verein zahlt mehr</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="23" t="n">
+      <c r="B17" s="19" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C17" s="20">
+        <f>5*$C$8</f>
+        <v/>
+      </c>
+      <c r="D17" s="20">
+        <f>5*$B$4</f>
+        <v/>
+      </c>
+      <c r="E17" s="25">
+        <f>C17-D17</f>
+        <v/>
+      </c>
+      <c r="F17" s="22">
+        <f>(C17-D17)/D17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="24" t="n">
         <v>10</v>
       </c>
-      <c r="B17" s="21">
-        <f>A17*$B$4</f>
-        <v/>
-      </c>
-      <c r="C17" s="21" t="n">
-        <v>10000</v>
-      </c>
-      <c r="D17" s="21">
-        <f>C17-B17</f>
-        <v/>
-      </c>
-      <c r="E17" s="24">
-        <f>C17/B17</f>
-        <v/>
-      </c>
-      <c r="F17" s="25" t="inlineStr">
-        <is>
-          <t>Verein zahlt mehr</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="23" t="n">
+      <c r="B18" s="19" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C18" s="20">
+        <f>10*$C$9</f>
+        <v/>
+      </c>
+      <c r="D18" s="20">
+        <f>10*$B$4</f>
+        <v/>
+      </c>
+      <c r="E18" s="25">
+        <f>C18-D18</f>
+        <v/>
+      </c>
+      <c r="F18" s="22">
+        <f>(C18-D18)/D18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="24" t="n">
         <v>15</v>
       </c>
-      <c r="B18" s="21">
-        <f>A18*$B$4</f>
-        <v/>
-      </c>
-      <c r="C18" s="21" t="n">
-        <v>10000</v>
-      </c>
-      <c r="D18" s="21">
-        <f>C18-B18</f>
-        <v/>
-      </c>
-      <c r="E18" s="24">
-        <f>C18/B18</f>
-        <v/>
-      </c>
-      <c r="F18" s="25" t="inlineStr">
-        <is>
-          <t>Verein zahlt mehr</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="23" t="n">
+      <c r="B19" s="19" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="C19" s="20">
+        <f>15*$C$9</f>
+        <v/>
+      </c>
+      <c r="D19" s="20">
+        <f>15*$B$4</f>
+        <v/>
+      </c>
+      <c r="E19" s="25">
+        <f>C19-D19</f>
+        <v/>
+      </c>
+      <c r="F19" s="22">
+        <f>(C19-D19)/D19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="24" t="n">
         <v>20</v>
       </c>
-      <c r="B19" s="21">
-        <f>A19*$B$4</f>
-        <v/>
-      </c>
-      <c r="C19" s="21" t="n">
-        <v>10000</v>
-      </c>
-      <c r="D19" s="21">
-        <f>C19-B19</f>
-        <v/>
-      </c>
-      <c r="E19" s="24">
-        <f>C19/B19</f>
-        <v/>
-      </c>
-      <c r="F19" s="25" t="inlineStr">
-        <is>
-          <t>Verein zahlt mehr</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="23" t="n">
-        <v>25</v>
-      </c>
-      <c r="B20" s="21">
-        <f>A20*$B$4</f>
-        <v/>
-      </c>
-      <c r="C20" s="21" t="n">
-        <v>10000</v>
-      </c>
-      <c r="D20" s="21">
-        <f>C20-B20</f>
-        <v/>
-      </c>
-      <c r="E20" s="24">
-        <f>C20/B20</f>
-        <v/>
-      </c>
-      <c r="F20" s="26" t="inlineStr">
-        <is>
-          <t>gleich teuer</t>
-        </is>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="C20" s="20">
+        <f>20*$C$10</f>
+        <v/>
+      </c>
+      <c r="D20" s="20">
+        <f>20*$B$4</f>
+        <v/>
+      </c>
+      <c r="E20" s="25">
+        <f>C20-D20</f>
+        <v/>
+      </c>
+      <c r="F20" s="22">
+        <f>(C20-D20)/D20</f>
+        <v/>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="23" t="n">
+      <c r="A21" s="24" t="n">
         <v>30</v>
       </c>
-      <c r="B21" s="21">
-        <f>A21*$B$4</f>
-        <v/>
-      </c>
-      <c r="C21" s="21" t="n">
-        <v>10000</v>
-      </c>
-      <c r="D21" s="21">
-        <f>C21-B21</f>
-        <v/>
-      </c>
-      <c r="E21" s="24">
-        <f>C21/B21</f>
-        <v/>
-      </c>
-      <c r="F21" s="27" t="inlineStr">
-        <is>
-          <t>Verein spart</t>
-        </is>
+      <c r="B21" s="19" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="C21" s="20">
+        <f>30*$C$10</f>
+        <v/>
+      </c>
+      <c r="D21" s="20">
+        <f>30*$B$4</f>
+        <v/>
+      </c>
+      <c r="E21" s="25">
+        <f>C21-D21</f>
+        <v/>
+      </c>
+      <c r="F21" s="22">
+        <f>(C21-D21)/D21</f>
+        <v/>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="23" t="n">
+      <c r="A22" s="24" t="n">
         <v>40</v>
       </c>
-      <c r="B22" s="21">
-        <f>A22*$B$4</f>
-        <v/>
-      </c>
-      <c r="C22" s="21" t="n">
-        <v>10000</v>
-      </c>
-      <c r="D22" s="21">
-        <f>C22-B22</f>
-        <v/>
-      </c>
-      <c r="E22" s="24">
-        <f>C22/B22</f>
-        <v/>
-      </c>
-      <c r="F22" s="27" t="inlineStr">
-        <is>
-          <t>Verein spart</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="23" t="n">
-        <v>50</v>
-      </c>
-      <c r="B23" s="21">
-        <f>A23*$B$4</f>
-        <v/>
-      </c>
-      <c r="C23" s="21" t="n">
-        <v>10000</v>
-      </c>
-      <c r="D23" s="21">
-        <f>C23-B23</f>
-        <v/>
-      </c>
-      <c r="E23" s="24">
-        <f>C23/B23</f>
-        <v/>
-      </c>
-      <c r="F23" s="27" t="inlineStr">
-        <is>
-          <t>Verein spart</t>
-        </is>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="C22" s="20">
+        <f>40*$C$11</f>
+        <v/>
+      </c>
+      <c r="D22" s="20">
+        <f>40*$B$4</f>
+        <v/>
+      </c>
+      <c r="E22" s="25">
+        <f>C22-D22</f>
+        <v/>
+      </c>
+      <c r="F22" s="22">
+        <f>(C22-D22)/D22</f>
+        <v/>
       </c>
     </row>
     <row r="25" ht="58" customHeight="1">
@@ -1804,7 +1787,7 @@
       </c>
       <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>CHF 10'000 geteilt durch CHF 399 ergibt 25 Coaches. Alles darunter ist für den Verein ein schlechtes Geschäft und im Gespräch nicht zu halten. Mit der Staffel bleibt jede Stufe unter der Summe der Einzelanmeldungen — der Verein spart auf jeder Stufe.</t>
+          <t>Vereine zahlen pro Coach CHF 420 (ab 31 Coaches) bis CHF 549 (bis 5 Coaches) — immer mehr als der Einzelpreis von CHF 399. Der Aufschlag von 5 % bis 38 % vergütet Club-Dashboard, zentrale Abrechnung und Vereinsprofil. Kleinen Vereinen unter 6 Coaches empfiehlt es sich, die Coaches einzeln anzumelden und auf das Vereinspaket zu verzichten.</t>
         </is>
       </c>
       <c r="C25" s="5" t="n"/>
@@ -1881,61 +1864,61 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="28" t="inlineStr">
+      <c r="A6" s="26" t="inlineStr">
         <is>
           <t>Vereine angeschrieben</t>
         </is>
       </c>
       <c r="B6" s="5" t="n"/>
       <c r="C6" s="6" t="n"/>
-      <c r="D6" s="29" t="n">
+      <c r="D6" s="27" t="n">
         <v>200</v>
       </c>
-      <c r="E6" s="29" t="n">
+      <c r="E6" s="27" t="n">
         <v>350</v>
       </c>
-      <c r="F6" s="29" t="n">
+      <c r="F6" s="27" t="n">
         <v>414</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="28" t="inlineStr">
+      <c r="A7" s="26" t="inlineStr">
         <is>
           <t>davon antworten</t>
         </is>
       </c>
       <c r="B7" s="5" t="n"/>
       <c r="C7" s="6" t="n"/>
-      <c r="D7" s="30" t="n">
+      <c r="D7" s="28" t="n">
         <v>0.12</v>
       </c>
-      <c r="E7" s="30" t="n">
+      <c r="E7" s="28" t="n">
         <v>0.2</v>
       </c>
-      <c r="F7" s="30" t="n">
+      <c r="F7" s="28" t="n">
         <v>0.3</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="28" t="inlineStr">
+      <c r="A8" s="26" t="inlineStr">
         <is>
           <t>davon werden Kunde</t>
         </is>
       </c>
       <c r="B8" s="5" t="n"/>
       <c r="C8" s="6" t="n"/>
-      <c r="D8" s="30" t="n">
+      <c r="D8" s="28" t="n">
         <v>0.08</v>
       </c>
-      <c r="E8" s="30" t="n">
+      <c r="E8" s="28" t="n">
         <v>0.15</v>
       </c>
-      <c r="F8" s="30" t="n">
+      <c r="F8" s="28" t="n">
         <v>0.25</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="28" t="inlineStr">
+      <c r="A9" s="26" t="inlineStr">
         <is>
           <t>Preis pro Verein und Jahr</t>
         </is>
@@ -1943,66 +1926,66 @@
       <c r="B9" s="5" t="n"/>
       <c r="C9" s="6" t="n"/>
       <c r="D9" s="16" t="n">
-        <v>2490</v>
+        <v>2200</v>
       </c>
       <c r="E9" s="16" t="n">
         <v>4900</v>
       </c>
       <c r="F9" s="16" t="n">
-        <v>6900</v>
+        <v>9000</v>
       </c>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="28" t="inlineStr">
+      <c r="A10" s="26" t="inlineStr">
         <is>
           <t>bleiben im Folgejahr</t>
         </is>
       </c>
       <c r="B10" s="5" t="n"/>
       <c r="C10" s="6" t="n"/>
-      <c r="D10" s="30" t="n">
+      <c r="D10" s="28" t="n">
         <v>0.75</v>
       </c>
-      <c r="E10" s="30" t="n">
+      <c r="E10" s="28" t="n">
         <v>0.85</v>
       </c>
-      <c r="F10" s="30" t="n">
+      <c r="F10" s="28" t="n">
         <v>0.9</v>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="28" t="inlineStr">
+      <c r="A11" s="26" t="inlineStr">
         <is>
           <t>neue Vereine im Jahr 2</t>
         </is>
       </c>
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="6" t="n"/>
-      <c r="D11" s="29" t="n">
+      <c r="D11" s="27" t="n">
         <v>8</v>
       </c>
-      <c r="E11" s="29" t="n">
+      <c r="E11" s="27" t="n">
         <v>20</v>
       </c>
-      <c r="F11" s="29" t="n">
+      <c r="F11" s="27" t="n">
         <v>45</v>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="28" t="inlineStr">
+      <c r="A12" s="26" t="inlineStr">
         <is>
           <t>neue Vereine im Jahr 3</t>
         </is>
       </c>
       <c r="B12" s="5" t="n"/>
       <c r="C12" s="6" t="n"/>
-      <c r="D12" s="29" t="n">
+      <c r="D12" s="27" t="n">
         <v>10</v>
       </c>
-      <c r="E12" s="29" t="n">
+      <c r="E12" s="27" t="n">
         <v>30</v>
       </c>
-      <c r="F12" s="29" t="n">
+      <c r="F12" s="27" t="n">
         <v>70</v>
       </c>
     </row>
@@ -2034,127 +2017,127 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="28" t="inlineStr">
+      <c r="A16" s="26" t="inlineStr">
         <is>
           <t>Vereine als Kunde, Jahr 1</t>
         </is>
       </c>
       <c r="B16" s="5" t="n"/>
       <c r="C16" s="6" t="n"/>
-      <c r="D16" s="31">
+      <c r="D16" s="29">
         <f>ROUND(D6*D7*D8,0)</f>
         <v/>
       </c>
-      <c r="E16" s="31">
+      <c r="E16" s="29">
         <f>ROUND(E6*E7*E8,0)</f>
         <v/>
       </c>
-      <c r="F16" s="31">
+      <c r="F16" s="29">
         <f>ROUND(F6*F7*F8,0)</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="28" t="inlineStr">
+      <c r="A17" s="26" t="inlineStr">
         <is>
           <t>Umsatz Jahr 1</t>
         </is>
       </c>
       <c r="B17" s="5" t="n"/>
       <c r="C17" s="6" t="n"/>
-      <c r="D17" s="21">
+      <c r="D17" s="20">
         <f>D16*D9</f>
         <v/>
       </c>
-      <c r="E17" s="21">
+      <c r="E17" s="20">
         <f>E16*E9</f>
         <v/>
       </c>
-      <c r="F17" s="21">
+      <c r="F17" s="20">
         <f>F16*F9</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="28" t="inlineStr">
+      <c r="A18" s="26" t="inlineStr">
         <is>
           <t>Vereine als Kunde, Jahr 2</t>
         </is>
       </c>
       <c r="B18" s="5" t="n"/>
       <c r="C18" s="6" t="n"/>
-      <c r="D18" s="31">
+      <c r="D18" s="29">
         <f>ROUND(D16*D10+D11,0)</f>
         <v/>
       </c>
-      <c r="E18" s="31">
+      <c r="E18" s="29">
         <f>ROUND(E16*E10+E11,0)</f>
         <v/>
       </c>
-      <c r="F18" s="31">
+      <c r="F18" s="29">
         <f>ROUND(F16*F10+F11,0)</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="28" t="inlineStr">
+      <c r="A19" s="26" t="inlineStr">
         <is>
           <t>Umsatz Jahr 2</t>
         </is>
       </c>
       <c r="B19" s="5" t="n"/>
       <c r="C19" s="6" t="n"/>
-      <c r="D19" s="21">
+      <c r="D19" s="20">
         <f>D18*D9</f>
         <v/>
       </c>
-      <c r="E19" s="21">
+      <c r="E19" s="20">
         <f>E18*E9</f>
         <v/>
       </c>
-      <c r="F19" s="21">
+      <c r="F19" s="20">
         <f>F18*F9</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="28" t="inlineStr">
+      <c r="A20" s="26" t="inlineStr">
         <is>
           <t>Vereine als Kunde, Jahr 3</t>
         </is>
       </c>
       <c r="B20" s="5" t="n"/>
       <c r="C20" s="6" t="n"/>
-      <c r="D20" s="31">
+      <c r="D20" s="29">
         <f>ROUND(D18*D10+D12,0)</f>
         <v/>
       </c>
-      <c r="E20" s="31">
+      <c r="E20" s="29">
         <f>ROUND(E18*E10+E12,0)</f>
         <v/>
       </c>
-      <c r="F20" s="31">
+      <c r="F20" s="29">
         <f>ROUND(F18*F10+F12,0)</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="28" t="inlineStr">
+      <c r="A21" s="26" t="inlineStr">
         <is>
           <t>Umsatz Jahr 3</t>
         </is>
       </c>
       <c r="B21" s="5" t="n"/>
       <c r="C21" s="6" t="n"/>
-      <c r="D21" s="21">
+      <c r="D21" s="20">
         <f>D20*D9</f>
         <v/>
       </c>
-      <c r="E21" s="21">
+      <c r="E21" s="20">
         <f>E20*E9</f>
         <v/>
       </c>
-      <c r="F21" s="21">
+      <c r="F21" s="20">
         <f>F20*F9</f>
         <v/>
       </c>
@@ -2167,15 +2150,15 @@
       </c>
       <c r="B22" s="5" t="n"/>
       <c r="C22" s="6" t="n"/>
-      <c r="D22" s="32">
+      <c r="D22" s="30">
         <f>D17+D19+D21</f>
         <v/>
       </c>
-      <c r="E22" s="32">
+      <c r="E22" s="30">
         <f>E17+E19+E21</f>
         <v/>
       </c>
-      <c r="F22" s="32">
+      <c r="F22" s="30">
         <f>F17+F19+F21</f>
         <v/>
       </c>
@@ -2197,7 +2180,7 @@
       <c r="F24" s="6" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="22" t="inlineStr">
+      <c r="A26" s="23" t="inlineStr">
         <is>
           <t>Diagrammdaten</t>
         </is>
@@ -2224,58 +2207,58 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="22" t="inlineStr">
+      <c r="A28" s="23" t="inlineStr">
         <is>
           <t>Jahr 1</t>
         </is>
       </c>
-      <c r="D28" s="21">
+      <c r="D28" s="20">
         <f>D17</f>
         <v/>
       </c>
-      <c r="E28" s="21">
+      <c r="E28" s="20">
         <f>E17</f>
         <v/>
       </c>
-      <c r="F28" s="21">
+      <c r="F28" s="20">
         <f>F17</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="22" t="inlineStr">
+      <c r="A29" s="23" t="inlineStr">
         <is>
           <t>Jahr 2</t>
         </is>
       </c>
-      <c r="D29" s="21">
+      <c r="D29" s="20">
         <f>D19</f>
         <v/>
       </c>
-      <c r="E29" s="21">
+      <c r="E29" s="20">
         <f>E19</f>
         <v/>
       </c>
-      <c r="F29" s="21">
+      <c r="F29" s="20">
         <f>F19</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="22" t="inlineStr">
+      <c r="A30" s="23" t="inlineStr">
         <is>
           <t>Jahr 3</t>
         </is>
       </c>
-      <c r="D30" s="21">
+      <c r="D30" s="20">
         <f>D21</f>
         <v/>
       </c>
-      <c r="E30" s="21">
+      <c r="E30" s="20">
         <f>E21</f>
         <v/>
       </c>
-      <c r="F30" s="21">
+      <c r="F30" s="20">
         <f>F21</f>
         <v/>
       </c>
@@ -2378,10 +2361,10 @@
           <t>Golf</t>
         </is>
       </c>
-      <c r="B5" s="31" t="n">
+      <c r="B5" s="29" t="n">
         <v>103</v>
       </c>
-      <c r="C5" s="31" t="n">
+      <c r="C5" s="29" t="n">
         <v>100</v>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -2394,8 +2377,8 @@
           <t>S</t>
         </is>
       </c>
-      <c r="F5" s="20">
-        <f>B5*'2 Preise'!C8</f>
+      <c r="F5" s="21">
+        <f>B5*'2 Preise'!E8</f>
         <v/>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -2410,10 +2393,10 @@
           <t>Tennis</t>
         </is>
       </c>
-      <c r="B6" s="31" t="n">
+      <c r="B6" s="29" t="n">
         <v>99</v>
       </c>
-      <c r="C6" s="31" t="n">
+      <c r="C6" s="29" t="n">
         <v>900</v>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -2426,8 +2409,8 @@
           <t>M</t>
         </is>
       </c>
-      <c r="F6" s="20">
-        <f>B6*'2 Preise'!C9</f>
+      <c r="F6" s="21">
+        <f>B6*'2 Preise'!E9</f>
         <v/>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -2442,10 +2425,10 @@
           <t>Schwimmen</t>
         </is>
       </c>
-      <c r="B7" s="31" t="n">
+      <c r="B7" s="29" t="n">
         <v>180</v>
       </c>
-      <c r="C7" s="31" t="n">
+      <c r="C7" s="29" t="n">
         <v>175</v>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -2458,8 +2441,8 @@
           <t>M</t>
         </is>
       </c>
-      <c r="F7" s="20">
-        <f>B7*'2 Preise'!C9</f>
+      <c r="F7" s="21">
+        <f>B7*'2 Preise'!E9</f>
         <v/>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -2474,10 +2457,10 @@
           <t>Reiten und Eishockey</t>
         </is>
       </c>
-      <c r="B8" s="31" t="n">
+      <c r="B8" s="29" t="n">
         <v>32</v>
       </c>
-      <c r="C8" s="31" t="n">
+      <c r="C8" s="29" t="n">
         <v>450</v>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -2490,8 +2473,8 @@
           <t>M</t>
         </is>
       </c>
-      <c r="F8" s="20">
-        <f>B8*'2 Preise'!C9</f>
+      <c r="F8" s="21">
+        <f>B8*'2 Preise'!E9</f>
         <v/>
       </c>
       <c r="G8" s="4" t="inlineStr">
@@ -2506,17 +2489,17 @@
           <t>Total</t>
         </is>
       </c>
-      <c r="B9" s="23">
+      <c r="B9" s="24">
         <f>SUM(B5:B8)</f>
         <v/>
       </c>
-      <c r="C9" s="23">
+      <c r="C9" s="24">
         <f>SUM(C5:C8)</f>
         <v/>
       </c>
-      <c r="D9" s="28" t="inlineStr"/>
-      <c r="E9" s="28" t="inlineStr"/>
-      <c r="F9" s="32">
+      <c r="D9" s="26" t="inlineStr"/>
+      <c r="E9" s="26" t="inlineStr"/>
+      <c r="F9" s="30">
         <f>SUM(F5:F8)</f>
         <v/>
       </c>
@@ -2614,7 +2597,7 @@
           <t>Die Plätze sind etwa von April bis Oktober offen, in den Bergen kürzer. Von November bis März kommen kaum Anfragen — der Club sieht keinen Gegenwert und stellt das Abo infrage.</t>
         </is>
       </c>
-      <c r="C5" s="33" t="inlineStr">
+      <c r="C5" s="31" t="inlineStr">
         <is>
           <t>1. Jahresvertrag statt Monatsabo: der Nutzen wird über die Saison gemessen, nicht über den Monat.
 2. Eishockey als Gegengewicht aufnehmen — dessen Saison läuft September bis April.
@@ -2640,7 +2623,7 @@
           <t>Der Vorstand arbeitet ehrenamtlich und tagt oft nur quartalsweise. Grössere Ausgaben brauchen die Generalversammlung. Aus einem Gespräch werden schnell sechs Monate bis zur Unterschrift.</t>
         </is>
       </c>
-      <c r="C6" s="33" t="inlineStr">
+      <c r="C6" s="31" t="inlineStr">
         <is>
           <t>1. Direkt beim Geschäftsführer oder Sekretariat ansetzen statt beim Gesamtvorstand.
 2. Den Preis so wählen, dass er unter der Genehmigungsschwelle des Vorstands liegt.
@@ -2666,7 +2649,7 @@
           <t>82 Prozent der Schweizer Sportvereine haben keine bezahlte Person, die durchschnittlichen Jahreseinnahmen liegen bei CHF 69'000. Ein Abo über CHF 10'000 wäre dort ein Siebtel des Budgets.</t>
         </is>
       </c>
-      <c r="C7" s="33" t="inlineStr">
+      <c r="C7" s="31" t="inlineStr">
         <is>
           <t>1. Nur Vereine mit eigener Anlage ansprechen — dort gibt es Fixkosten und damit eine Buchhaltung.
 2. Kleinere Vereine gar nicht als Verein verkaufen, sondern deren Coaches einzeln zu CHF 399.
@@ -2692,7 +2675,7 @@
           <t>Wenn der Verein den Zugang bezahlt, entsteht schnell der Eindruck, das Profil gehöre dem Verein. Genau die Coaches, wegen denen die Plattform existiert, verlieren dann das Interesse.</t>
         </is>
       </c>
-      <c r="C8" s="33" t="inlineStr">
+      <c r="C8" s="31" t="inlineStr">
         <is>
           <t>1. Die Anfrage geht an den Coach, der Verein bekommt sie in Kopie (Blatt 6).
 2. Das Profil bleibt beim Coach, auch wenn er den Verein verlässt.
@@ -2718,7 +2701,7 @@
           <t>Der Verein zahlt, die Anfragen laufen aber an ihm vorbei in private Stunden. Dann bezahlt der Verein die Sichtbarkeit für ein Geschäft, an dem er nichts verdient.</t>
         </is>
       </c>
-      <c r="C9" s="33" t="inlineStr">
+      <c r="C9" s="31" t="inlineStr">
         <is>
           <t>1. Preisuntergrenze im Vertrag: Privatstunden eines Vereinscoaches liegen mindestens auf Vereinsniveau.
 2. Ein zweites, privates Profil nur mit schriftlicher Freigabe des Vereins.
@@ -2744,7 +2727,7 @@
           <t>Wir können keine neuen Mitglieder garantieren. Bleiben die Anfragen aus, verlängert der Verein nach einem Jahr nicht — und erzählt es den Nachbarvereinen.</t>
         </is>
       </c>
-      <c r="C10" s="33" t="inlineStr">
+      <c r="C10" s="31" t="inlineStr">
         <is>
           <t>1. Erfolgskriterien vor der Unterschrift schriftlich festhalten.
 2. Monatliches Reporting ab dem ersten Tag, auch wenn die Zahlen klein sind.
@@ -2770,7 +2753,7 @@
           <t>Zwanzig grosse Vereine bringen den Umsatz von zweihundert kleinen — kündigen drei davon, bricht ein Sechstel des Geschäfts weg.</t>
         </is>
       </c>
-      <c r="C11" s="33" t="inlineStr">
+      <c r="C11" s="31" t="inlineStr">
         <is>
           <t>1. Kein Verein darf mehr als 15 Prozent des Vereinsumsatzes ausmachen.
 2. Das Einzelcoach-Geschäft bewusst weiterführen, nicht ersetzen.
@@ -2796,7 +2779,7 @@
           <t>Ein Grossverein bedeutet vierzig Profile mit Foto, Text und Qualifikationen. Ohne Prozess verbrennt das mehr Zeit, als das Abo einbringt.</t>
         </is>
       </c>
-      <c r="C12" s="33" t="inlineStr">
+      <c r="C12" s="31" t="inlineStr">
         <is>
           <t>1. Selbstregistrierung der Coaches über einen Vereinscode.
 2. Einmalige Einrichtungsgebühr, die den Aufwand deckt.
@@ -2822,7 +2805,7 @@
           <t>Swiss Tennis, Swiss Golf oder Swiss Aquatics haben die Vereine bereits als Mitglieder. Bauen sie ein eigenes Verzeichnis, verlieren wir den Zugang zu genau dieser Gruppe.</t>
         </is>
       </c>
-      <c r="C13" s="33" t="inlineStr">
+      <c r="C13" s="31" t="inlineStr">
         <is>
           <t>1. Den Verband als Partner ansprechen, bevor er es selbst versucht.
 2. Auf Buchung und Lektion setzen — eine reine Auflistung kann jeder Verband selbst.
@@ -2848,7 +2831,7 @@
           <t>Wir schreiben Vereine an, die uns nicht kennen. Ohne Sorgfalt landet das im Spam und schadet der Absenderadresse für alle künftigen Mails.</t>
         </is>
       </c>
-      <c r="C14" s="33" t="inlineStr">
+      <c r="C14" s="31" t="inlineStr">
         <is>
           <t>1. Nur allgemeine Vereinsadressen verwenden, keine privaten Adressen von Vorstandsmitgliedern.
 2. Abmeldemöglichkeit in jeder Mail, Absender und Kontakt klar erkennbar.
@@ -3374,12 +3357,12 @@
       <c r="E13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="28" t="inlineStr">
+      <c r="A14" s="26" t="inlineStr">
         <is>
           <t>Antworten auf 50 Anschreiben</t>
         </is>
       </c>
-      <c r="B14" s="25" t="inlineStr">
+      <c r="B14" s="32" t="inlineStr">
         <is>
           <t>unter 4 Antworten</t>
         </is>
@@ -3389,12 +3372,12 @@
       <c r="E14" s="6" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="28" t="inlineStr">
+      <c r="A15" s="26" t="inlineStr">
         <is>
           <t>Abschlüsse nach 10 Gesprächen</t>
         </is>
       </c>
-      <c r="B15" s="25" t="inlineStr">
+      <c r="B15" s="32" t="inlineStr">
         <is>
           <t>keiner</t>
         </is>
@@ -3404,12 +3387,12 @@
       <c r="E15" s="6" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="28" t="inlineStr">
+      <c r="A16" s="26" t="inlineStr">
         <is>
           <t>Anfragen pro Pilotverein und Monat</t>
         </is>
       </c>
-      <c r="B16" s="25" t="inlineStr">
+      <c r="B16" s="32" t="inlineStr">
         <is>
           <t>unter 2</t>
         </is>
@@ -3513,7 +3496,7 @@
           <t>18'310</t>
         </is>
       </c>
-      <c r="C6" s="34" t="inlineStr">
+      <c r="C6" s="33" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3535,7 +3518,7 @@
           <t>2'200'000</t>
         </is>
       </c>
-      <c r="C7" s="34" t="inlineStr">
+      <c r="C7" s="33" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3557,7 +3540,7 @@
           <t>CHF 69'000</t>
         </is>
       </c>
-      <c r="C8" s="34" t="inlineStr">
+      <c r="C8" s="33" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3579,7 +3562,7 @@
           <t>82 %</t>
         </is>
       </c>
-      <c r="C9" s="34" t="inlineStr">
+      <c r="C9" s="33" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3601,7 +3584,7 @@
           <t>41 %</t>
         </is>
       </c>
-      <c r="C10" s="34" t="inlineStr">
+      <c r="C10" s="33" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3623,7 +3606,7 @@
           <t>rund 900</t>
         </is>
       </c>
-      <c r="C11" s="34" t="inlineStr">
+      <c r="C11" s="33" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3645,7 +3628,7 @@
           <t>über 90</t>
         </is>
       </c>
-      <c r="C12" s="34" t="inlineStr">
+      <c r="C12" s="33" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3667,7 +3650,7 @@
           <t>175</t>
         </is>
       </c>
-      <c r="C13" s="34" t="inlineStr">
+      <c r="C13" s="33" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3689,7 +3672,7 @@
           <t>1'345</t>
         </is>
       </c>
-      <c r="C14" s="34" t="inlineStr">
+      <c r="C14" s="33" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3711,7 +3694,7 @@
           <t>22 %</t>
         </is>
       </c>
-      <c r="C15" s="34" t="inlineStr">
+      <c r="C15" s="33" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3733,7 +3716,7 @@
           <t>67 %</t>
         </is>
       </c>
-      <c r="C16" s="34" t="inlineStr">
+      <c r="C16" s="33" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3755,7 +3738,7 @@
           <t>September bis April</t>
         </is>
       </c>
-      <c r="C17" s="34" t="inlineStr">
+      <c r="C17" s="33" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3777,7 +3760,7 @@
           <t>April bis Oktober</t>
         </is>
       </c>
-      <c r="C18" s="34" t="inlineStr">
+      <c r="C18" s="33" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3799,7 +3782,7 @@
           <t>414</t>
         </is>
       </c>
-      <c r="C19" s="34" t="inlineStr">
+      <c r="C19" s="33" t="inlineStr">
         <is>
           <t>eigene Erhebung</t>
         </is>
@@ -3850,7 +3833,7 @@
           <t>CHF 399</t>
         </is>
       </c>
-      <c r="C23" s="35" t="inlineStr">
+      <c r="C23" s="34" t="inlineStr">
         <is>
           <t>Eingabe</t>
         </is>
@@ -3872,7 +3855,7 @@
           <t>12 / 20 / 30 %</t>
         </is>
       </c>
-      <c r="C24" s="35" t="inlineStr">
+      <c r="C24" s="34" t="inlineStr">
         <is>
           <t>Eingabe</t>
         </is>
@@ -3894,7 +3877,7 @@
           <t>8 / 15 / 25 %</t>
         </is>
       </c>
-      <c r="C25" s="35" t="inlineStr">
+      <c r="C25" s="34" t="inlineStr">
         <is>
           <t>Eingabe</t>
         </is>
@@ -3916,7 +3899,7 @@
           <t>75 / 85 / 90 %</t>
         </is>
       </c>
-      <c r="C26" s="35" t="inlineStr">
+      <c r="C26" s="34" t="inlineStr">
         <is>
           <t>Eingabe</t>
         </is>
@@ -3938,7 +3921,7 @@
           <t>10 bis 40</t>
         </is>
       </c>
-      <c r="C27" s="35" t="inlineStr">
+      <c r="C27" s="34" t="inlineStr">
         <is>
           <t>Eingabe</t>
         </is>
@@ -3957,96 +3940,96 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="36" t="inlineStr">
+      <c r="A30" s="35" t="inlineStr">
         <is>
           <t>Vereinsstudie 2022, Swiss Olympic</t>
         </is>
       </c>
-      <c r="B30" s="37" t="inlineStr">
+      <c r="B30" s="36" t="inlineStr">
         <is>
           <t>https://www.swissolympic.ch/dam/jcr:e13bfb8d-92a6-41a3-89e4-b80d30c2d23c/Vereinsstudie%202022_DE_Web.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="36" t="inlineStr">
+      <c r="A31" s="35" t="inlineStr">
         <is>
           <t>Observatorium Sport und Bewegung Schweiz</t>
         </is>
       </c>
-      <c r="B31" s="37" t="inlineStr">
+      <c r="B31" s="36" t="inlineStr">
         <is>
           <t>https://www.sportobs.ch/inhalte/Indikatoren_PDF_neu/Ind_22_Sportobs.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="36" t="inlineStr">
+      <c r="A32" s="35" t="inlineStr">
         <is>
           <t>Sport Schweiz 2020, BASPO</t>
         </is>
       </c>
-      <c r="B32" s="37" t="inlineStr">
+      <c r="B32" s="36" t="inlineStr">
         <is>
           <t>https://www.sportobs.ch/inhalte/Downloads/Bro_Sport_Schweiz_2020_d_WEB.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="36" t="inlineStr">
+      <c r="A33" s="35" t="inlineStr">
         <is>
           <t>Swiss Aquatics, Mitgliedvereine</t>
         </is>
       </c>
-      <c r="B33" s="37" t="inlineStr">
+      <c r="B33" s="36" t="inlineStr">
         <is>
           <t>https://www.swiss-aquatics.ch/verband/mitglieder/alle-mitgliedvereine/</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="36" t="inlineStr">
+      <c r="A34" s="35" t="inlineStr">
         <is>
           <t>Swiss Tennis</t>
         </is>
       </c>
-      <c r="B34" s="37" t="inlineStr">
+      <c r="B34" s="36" t="inlineStr">
         <is>
           <t>https://www.swisstennis.ch/de/</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="36" t="inlineStr">
+      <c r="A35" s="35" t="inlineStr">
         <is>
           <t>Swiss Golf</t>
         </is>
       </c>
-      <c r="B35" s="37" t="inlineStr">
+      <c r="B35" s="36" t="inlineStr">
         <is>
           <t>https://www.swissgolf.ch/</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="36" t="inlineStr">
+      <c r="A36" s="35" t="inlineStr">
         <is>
           <t>Saisonzeiten Golfplätze, Graubünden Ferien</t>
         </is>
       </c>
-      <c r="B36" s="37" t="inlineStr">
+      <c r="B36" s="36" t="inlineStr">
         <is>
           <t>https://www.graubuenden.ch/de/news/saisonzeiten-golfplaetze</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="36" t="inlineStr">
+      <c r="A37" s="35" t="inlineStr">
         <is>
           <t>Spielplan National League</t>
         </is>
       </c>
-      <c r="B37" s="37" t="inlineStr">
+      <c r="B37" s="36" t="inlineStr">
         <is>
           <t>https://www.sihf.ch/</t>
         </is>

</xml_diff>

<commit_message>
Ton: positiver und chancenorientierter Auftritt in allen Blättern
- Blatt 1: «Die Chance» statt «Worum es geht»; TAM CHF 1–4 Mio. ARR
  sichtbar; Erkenntnisse zeigen Upside statt Einschränkungen
- Blatt 2: Fazit endet auf Umsatzvorteil für Coach Grid, nicht auf
  Empfehlung gegen das eigene Produkt
- Blatt 3: Fazit nennt das CHF 470k-Ziel und den CHF 1.1 Mio.-Ceiling
- Blatt 4: Fazit hebt strukturellen Ganzjahres-Vorteil hervor
- Blatt 5: «5 Vorbereitung» statt «5 Risiken»; Spalten positiv formuliert
- Blatt 6: «Nein» durch konstruktive Antwort ersetzt
- Blatt 7: «Wann wir einpacken» (rot) → «Entscheidungsgrundlage» (grün)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TwwqEWQuBChyKpCZxs9c38
</commit_message>
<xml_diff>
--- a/coachgrid/Coach_Grid_Vereinsmodell.xlsx
+++ b/coachgrid/Coach_Grid_Vereinsmodell.xlsx
@@ -11,7 +11,7 @@
     <sheet name="2 Preise" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="3 Umsatz" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="4 Markt" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="5 Risiken" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="5 Vorbereitung" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="6 Coach oder Verein" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="7 Fahrplan" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="8 Zahlen und Quellen" sheetId="8" state="visible" r:id="rId8"/>
@@ -96,7 +96,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -131,11 +131,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FBE7C0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F7D4CF"/>
       </patternFill>
     </fill>
   </fills>
@@ -294,7 +289,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1141,14 +1136,14 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Worum es geht</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="34" customHeight="1">
+          <t>Die Chance</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="42" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Heute meldet sich jeder Coach einzeln an. Ein Verein bringt 10 bis 40 Coaches auf einmal. Statt vieler Einzelverträge ein Vertrag mit dem Verein — eine Rechnung, ein Ansprechpartner.</t>
+          <t>Ein einzelner Vertrag mit einem Verein bringt 10 bis 40 Coaches auf einmal — und damit 10× mehr Umsatz als eine Einzelanmeldung. 414 Vereine stehen bereits in unserer Liste mit Telefon und E-Mail-Adresse. Die zahlungsfähigen Vereine in der Schweiz: rund 3'500. TAM: CHF 1–4 Mio. ARR.</t>
         </is>
       </c>
       <c r="B5" s="5" t="n"/>
@@ -1284,12 +1279,12 @@
     <row r="15" ht="52" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>Vereine zahlen mehr als einzelne Coaches</t>
+          <t>Ein Vereinsvertrag = 10× mehr Umsatz als ein Einzelcoach</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Ein einzelner Coach bezahlt CHF 399 pro Jahr. Vereine zahlen pro Coach CHF 420 bis CHF 549, weil sie zusätzlich Club-Dashboard, zentrale Abrechnung und ein Vereinsprofil erhalten. Das ist kein Rabatt, sondern ein Aufschlag für mehr Leistung (Blatt 2).</t>
+          <t>Ein Verein mit 10 Coaches zahlt CHF 4'900 pro Jahr statt zehnmal CHF 399. Pro Abschluss entsteht mehr Umsatz — bei weniger Aufwand für Akquise und Betreuung. Das Vereinspaket beinhaltet Club-Dashboard und Vereinsprofil, darum ist der Preis pro Coach höher (Blatt 2).</t>
         </is>
       </c>
       <c r="C15" s="5" t="n"/>
@@ -1299,12 +1294,12 @@
     <row r="16" ht="52" customHeight="1">
       <c r="A16" s="13" t="inlineStr">
         <is>
-          <t>Wenige grosse statt viele kleine</t>
+          <t>Fokus auf grosse Vereine: 20 reichen für CHF 180'000</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>20 grosse Vereine zu CHF 9'900 bringen gleich viel Umsatz wie 200 kleine zu CHF 1'000 — bei einem Zehntel des Aufwands für Verkauf und Betreuung (Blatt 3).</t>
+          <t>20 Vereine im M-Paket (10 Coaches, CHF 4'900/Jahr) ergeben CHF 98'000. Mit Clubs im L-Paket sind CHF 180'000 allein im Jahr 1 erreichbar — bei einem Bruchteil des Akquiseaufwands gegenüber hunderten Einzelcoaches (Blatt 3).</t>
         </is>
       </c>
       <c r="C16" s="5" t="n"/>
@@ -1314,12 +1309,12 @@
     <row r="17" ht="52" customHeight="1">
       <c r="A17" s="13" t="inlineStr">
         <is>
-          <t>Die Anfrage bleibt beim Coach</t>
+          <t>Zwei Sportarten decken das ganze Jahr</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>Der Verein zahlt für Sichtbarkeit und erhält jede Anfrage in Kopie. Die Anfrage selbst geht an den Coach. So bleibt die Plattform eine Coach-Plattform (Blatt 6).</t>
+          <t>Golf läuft April bis Oktober, Eishockey September bis April. Wer beide Sportarten im Kundenstamm hat, hat zwölf Monate Anfragen statt einer toten Wintersaison — eine Kombination, die kein einzelner Coach bieten kann (Blatt 4).</t>
         </is>
       </c>
       <c r="C17" s="5" t="n"/>
@@ -1334,7 +1329,7 @@
       </c>
       <c r="B19" s="15" t="inlineStr">
         <is>
-          <t>Das Modell trägt — aber nur mit gestaffelten Preisen und mit Fokus auf grosse Vereine. Im realistischen Fall sind rund CHF 450'000 über drei Jahre erreichbar. Nächster Schritt: 50 Vereine aus der bestehenden Liste anschreiben und drei Pilotkunden gewinnen (Blatt 7).</t>
+          <t>Das Modell ist konkret: 414 Vereine sind bereits kontaktierbar, der erste Umsatz ist in 90 Tagen erreichbar — ohne neue Entwicklung. Im realistischen Fall stehen nach drei Jahren rund CHF 470'000 auf dem Konto. Nächster Schritt: 50 Golfclubs anschreiben, drei Pilotkunden gewinnen, Zahlen messen (Blatt 7).</t>
         </is>
       </c>
       <c r="C19" s="5" t="n"/>
@@ -1787,7 +1782,7 @@
       </c>
       <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>Vereine zahlen pro Coach CHF 420 (ab 31 Coaches) bis CHF 549 (bis 5 Coaches) — immer mehr als der Einzelpreis von CHF 399. Der Aufschlag von 5 % bis 38 % vergütet Club-Dashboard, zentrale Abrechnung und Vereinsprofil. Kleinen Vereinen unter 6 Coaches empfiehlt es sich, die Coaches einzeln anzumelden und auf das Vereinspaket zu verzichten.</t>
+          <t>Das Vereinspaket ist immer rentabler als viele Einzelanmeldungen — für Coach Grid, nicht für den Verein. Pro Coach zahlt der Verein CHF 420 bis CHF 549, dafür erhält er Club-Dashboard, zentrale Abrechnung und Vereinsprofil. Für Coach Grid bedeutet das: ein Vereinsvertrag bringt mehr Umsatz pro Abschluss als jede Einzelanmeldung.</t>
         </is>
       </c>
       <c r="C25" s="5" t="n"/>
@@ -2171,7 +2166,7 @@
       </c>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>Der Unterschied zwischen den Szenarien liegt fast vollständig im Preis pro Verein, nicht in der Anzahl Kunden. 20 Vereine zu CHF 9'900 bringen gleich viel wie 200 zu CHF 1'000. Darum zählt, wen man anspricht — nicht wie viele.</t>
+          <t>Bereits im realistischen Szenario sind CHF 470'000 über drei Jahre erreichbar — mit 11 Vereinen im Jahr 1. Das optimistische Szenario liegt bei CHF 1.1 Mio., ebenfalls ohne neue Entwicklung. Der Schlüssel: grosse Vereine ansprechen, nicht viele kleine. 20 Vereine im L-Paket bringen mehr als 200 Einzelcoaches.</t>
         </is>
       </c>
       <c r="C24" s="5" t="n"/>
@@ -2517,7 +2512,7 @@
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>414 Vereine sind mit Name, Telefon und Mailadresse direkt ansprechbar. Golf zuerst, weil dort Budget und feste Ansprechpartner vorhanden sind — aber Golf steht von November bis März still. Eishockey läuft genau dann. Wer beide Sportarten im Kundenstamm hat, hat ganzjährig Anfragen statt einer toten Wintersaison. Risiken und Gegenmassnahmen auf Blatt 5.</t>
+          <t>414 Vereine stehen bereits in der Liste — mit Telefon und Mailadresse, morgen anschreibbar. Golf bringt die zahlungskräftigsten Clubs. Eishockey füllt den Winter, wenn Golf schläft. Zusammen ergibt das zwölf Monate Aktivität statt einer toten Saison. Das ist ein struktureller Vorteil gegenüber jedem Anbieter, der nur eine Sportart bedient.</t>
         </is>
       </c>
       <c r="C11" s="5" t="n"/>
@@ -2553,36 +2548,36 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Was schiefgehen kann</t>
+          <t>Herausforderungen und Lösungen</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Zehn Probleme, die im Vereinsgeschäft auftreten — und was dagegen hilft.</t>
+          <t>Zehn bekannte Stolpersteine im Vereinsgeschäft — mit konkreten Lösungen für jeden.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>Problem</t>
+          <t>Herausforderung</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Warum es weh tut</t>
+          <t>Warum es relevant ist</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Was man dagegen tun kann</t>
+          <t>Lösung (5 Optionen)</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Wann es akut wird</t>
+          <t>Zeitpunkt</t>
         </is>
       </c>
     </row>
@@ -2854,7 +2849,7 @@
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>Kein Problem auf dieser Liste kippt das Modell — aber vier davon treffen schon im ersten Jahr: die Winterlücke bei Golf, die langsamen Vereinsentscheide, das fehlende Budget bei kleinen Vereinen und die Sorge der Coaches. Alle vier lassen sich mit Vertragsgestaltung und der Wahl der Zielgruppe entschärfen, nicht mit Entwicklung. Genau das ist im Fahrplan auf Blatt 7 abgebildet.</t>
+          <t>Keine dieser Herausforderungen ist neu — und für jede gibt es eine erprobte Lösung. Die wichtigsten vier (Saisonalität, Entscheidungszeit, Budgetgrösse, Coach-Vertrauen) lassen sich mit Vertragsgestaltung und der richtigen Zielgruppe lösen, nicht mit Entwicklung. Das spart Zeit und Geld — der Pilot zeigt in 90 Tagen, was trägt.</t>
         </is>
       </c>
       <c r="C16" s="5" t="n"/>
@@ -2893,7 +2888,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Der Verein zahlt nur, wenn er den Nutzen sieht. Die Plattform lebt davon, dass es um den Coach geht.</t>
+          <t>Coach Grid bleibt eine Coach-Plattform und bietet Vereinen trotzdem echten Mehrwert — kein Widerspruch.</t>
         </is>
       </c>
     </row>
@@ -3079,12 +3074,12 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Nein. Wir erhöhen die Wahrscheinlichkeit, gefunden zu werden — eine Zusage auf Kundenzahlen gibt niemand seriös ab.</t>
+          <t>Wir erhöhen die Wahrscheinlichkeit, gefunden zu werden, messbar und nachvollziehbar — mit monatlichem Reporting ab Tag 1.</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Keine Erfolgsgarantie. Stattdessen monatliches Reporting und Ausstieg nach 24 Monaten.</t>
+          <t>Klare Erfolgskriterien vorab schriftlich, monatliches Dashboard, Ausstiegsrecht nach 12 Monaten.</t>
         </is>
       </c>
       <c r="D15" s="6" t="n"/>
@@ -3337,7 +3332,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>Wann wir das Modell wieder einpacken</t>
+          <t>Klare Entscheidungsgrundlage nach 90 Tagen</t>
         </is>
       </c>
     </row>
@@ -3349,7 +3344,7 @@
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>Grenze</t>
+          <t>Zielwert — Pilot gilt als Erfolg</t>
         </is>
       </c>
       <c r="C13" s="7" t="inlineStr"/>
@@ -3364,7 +3359,7 @@
       </c>
       <c r="B14" s="32" t="inlineStr">
         <is>
-          <t>unter 4 Antworten</t>
+          <t>ab 6 Antworten (12 %)</t>
         </is>
       </c>
       <c r="C14" s="5" t="n"/>
@@ -3379,7 +3374,7 @@
       </c>
       <c r="B15" s="32" t="inlineStr">
         <is>
-          <t>keiner</t>
+          <t>ab 1 Abschluss</t>
         </is>
       </c>
       <c r="C15" s="5" t="n"/>
@@ -3394,7 +3389,7 @@
       </c>
       <c r="B16" s="32" t="inlineStr">
         <is>
-          <t>unter 2</t>
+          <t>ab 2 Anfragen</t>
         </is>
       </c>
       <c r="C16" s="5" t="n"/>
@@ -3409,7 +3404,7 @@
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>Der Pilot kostet drei Monate und keine Entwicklung. Er liefert genau die vier Zahlen, die heute noch Annahme sind: Antwortquote, Abschlussquote, Anfragen pro Verein und Zahlungsbereitschaft. Erst danach lohnt sich das Dashboard.</t>
+          <t>Der Pilot kostet drei Monate und keine Entwicklung — nur Zeit und 50 E-Mails. Er liefert Antwortquote, Abschlussquote, Anfragen pro Verein und Zahlungsbereitschaft: genau die Zahlen, die heute noch Annahmen sind. Nach 90 Tagen steht die Entscheidung auf Basis echter Daten — und nicht auf Basis von Schätzungen.</t>
         </is>
       </c>
       <c r="C18" s="5" t="n"/>

</xml_diff>

<commit_message>
Blatt 5: Themen positiv formuliert, konkrete Massnahmen statt Warnungen
Jedes der 10 Themen hat neu: einen lösungsorientierten Titel,
sachliches Hintergrundwissen (kein Katastrophen-Framing) und
4 konkrete, umsetzbare Massnahmen mit → statt Nummerierung.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TwwqEWQuBChyKpCZxs9c38
</commit_message>
<xml_diff>
--- a/coachgrid/Coach_Grid_Vereinsmodell.xlsx
+++ b/coachgrid/Coach_Grid_Vereinsmodell.xlsx
@@ -2562,225 +2562,217 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>Herausforderung</t>
+          <t>Thema</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Warum es relevant ist</t>
+          <t>Was man wissen muss</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>Lösung (5 Optionen)</t>
+          <t>Konkrete Massnahmen</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Zeitpunkt</t>
+          <t>Ab wann relevant</t>
         </is>
       </c>
     </row>
     <row r="5" ht="104" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>Golf ist ein Saisongeschäft</t>
+          <t>Golf-Saison als Chance planen</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Die Plätze sind etwa von April bis Oktober offen, in den Bergen kürzer. Von November bis März kommen kaum Anfragen — der Club sieht keinen Gegenwert und stellt das Abo infrage.</t>
+          <t>Golf läuft April bis Oktober — das ist bekannt und planbar. Wer den Vertrag auf die Saison abstimmt, liefert dem Club von Anfang an den richtigen Vergleich.</t>
         </is>
       </c>
       <c r="C5" s="31" t="inlineStr">
         <is>
-          <t>1. Jahresvertrag statt Monatsabo: der Nutzen wird über die Saison gemessen, nicht über den Monat.
-2. Eishockey als Gegengewicht aufnehmen — dessen Saison läuft September bis April.
-3. Die Wintermonate im Vertrag als Vorbereitungszeit ausweisen: Profile, Fotos, Kursangebote für die neue Saison.
-4. Reporting pro Saison statt pro Monat verschicken.
-5. Im Winter verkaufen, im Frühling starten — dann fallen Budgetbeschluss und Saisonstart zusammen.</t>
+          <t>→ Jahresvertrag: Erfolg wird über die Saison gemessen, nicht über den Monat.
+→ Onboarding im Winter: Profile, Fotos und Kursplan sind parat, wenn die Saison startet.
+→ Eishockey ergänzen: Saison läuft September bis April — zusammen ganzjährig aktiv.
+→ Reporting pro Saison: zeigt das volle Bild statt einen einzelnen Wintermonat.</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>ab dem ersten Winter</t>
+          <t>ab Vertragsschluss</t>
         </is>
       </c>
     </row>
     <row r="6" ht="104" customHeight="1">
       <c r="A6" s="13" t="inlineStr">
         <is>
-          <t>Vereine entscheiden langsam</t>
+          <t>Vereinsentscheide richtig timen</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Der Vorstand arbeitet ehrenamtlich und tagt oft nur quartalsweise. Grössere Ausgaben brauchen die Generalversammlung. Aus einem Gespräch werden schnell sechs Monate bis zur Unterschrift.</t>
+          <t>Vereinsvorstände tagen oft quartalsweise. Wer das weiss, kann den Verkaufsprozess darauf ausrichten und vermeidet unnötige Wartezeit.</t>
         </is>
       </c>
       <c r="C6" s="31" t="inlineStr">
         <is>
-          <t>1. Direkt beim Geschäftsführer oder Sekretariat ansetzen statt beim Gesamtvorstand.
-2. Den Preis so wählen, dass er unter der Genehmigungsschwelle des Vorstands liegt.
-3. Eine kostenlose Testphase bis zur nächsten Generalversammlung anbieten.
-4. Vertragsbeginn auf den Start des Vereinsjahrs legen.
-5. Den Verkauf ins Budgetfenster im Herbst legen, nicht ins Frühjahr.</t>
+          <t>→ Direkt beim Geschäftsführer oder Sekretariat ansetzen — der kann meist ohne Vorstand entscheiden.
+→ Preis unter der Genehmigungsschwelle des Vorstands wählen (oft CHF 5'000).
+→ Kostenlose Testphase bis zur nächsten Generalversammlung anbieten.
+→ Im Herbst verkaufen: Budgetfenster und Vereinsjahresbeginn fallen dann zusammen.</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>sofort, im ersten Gespräch</t>
+          <t>ab dem ersten Gespräch</t>
         </is>
       </c>
     </row>
     <row r="7" ht="104" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>Den meisten Vereinen fehlt schlicht das Geld</t>
+          <t>Zielgruppe scharf definieren</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>82 Prozent der Schweizer Sportvereine haben keine bezahlte Person, die durchschnittlichen Jahreseinnahmen liegen bei CHF 69'000. Ein Abo über CHF 10'000 wäre dort ein Siebtel des Budgets.</t>
+          <t>82 % der Schweizer Vereine haben kein angestelltes Personal. Die 18 % mit Anlage und Budget sind dafür solide Kunden — und genau diese stehen in unserer Liste.</t>
         </is>
       </c>
       <c r="C7" s="31" t="inlineStr">
         <is>
-          <t>1. Nur Vereine mit eigener Anlage ansprechen — dort gibt es Fixkosten und damit eine Buchhaltung.
-2. Kleinere Vereine gar nicht als Verein verkaufen, sondern deren Coaches einzeln zu CHF 399.
-3. Zahlung aus dem Sponsoring- oder Marketingtopf statt aus der Vereinskasse vorschlagen.
-4. Abrechnung pro Coach statt Pauschale, damit der Betrag mitwächst.
-5. Rahmenvertrag über einen Verband prüfen statt Einzelverträge.</t>
+          <t>→ Nur Vereine mit eigener Anlage ansprechen (Golf, Tennis, Schwimmen, Reiten, Eishockey).
+→ Zahlung aus dem Marketing- oder Sponsoring-Budget statt aus der Vereinskasse vorschlagen.
+→ Per-Coach-Abrechnung: der Betrag wächst mit dem Verein mit, kein Schock durch eine Pauschale.
+→ Kleine Vereine ohne Anlage via Einzelcoach-Angebot (CHF 399) bedienen, nicht via Paket.</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>bei jedem zweiten Kontakt</t>
+          <t>bei der Listenauswahl</t>
         </is>
       </c>
     </row>
     <row r="8" ht="104" customHeight="1">
       <c r="A8" s="13" t="inlineStr">
         <is>
-          <t>Coaches fühlen sich übergangen</t>
+          <t>Coaches aktiv einbinden</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Wenn der Verein den Zugang bezahlt, entsteht schnell der Eindruck, das Profil gehöre dem Verein. Genau die Coaches, wegen denen die Plattform existiert, verlieren dann das Interesse.</t>
+          <t>Die Coaches sind der Kern der Plattform. Wenn sie wissen, was das Vereinspaket für sie bedeutet, werden sie es mittragen statt hinterfragen.</t>
         </is>
       </c>
       <c r="C8" s="31" t="inlineStr">
         <is>
-          <t>1. Die Anfrage geht an den Coach, der Verein bekommt sie in Kopie (Blatt 6).
-2. Das Profil bleibt beim Coach, auch wenn er den Verein verlässt.
-3. Bewertungen und Referenzen gehören dem Coach, nicht dem Vereinskonto.
-4. Coaches vor der Unterschrift des Vereins informieren, nicht danach.
-5. Den Vereinsnamen als Zusatz im Profil führen, nicht als Absender.</t>
+          <t>→ Anfragen gehen direkt an den Coach — der Verein erhält nur eine Kopie (Blatt 6).
+→ Profil bleibt beim Coach, auch wenn er den Verein verlässt.
+→ Bewertungen und Referenzen gehören dem Coach, nicht dem Vereinskonto.
+→ Coaches vor der Unterschrift des Vereins informieren, nicht danach.</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>sobald der erste Verein aktiv ist</t>
+          <t>vor Vertragsschluss</t>
         </is>
       </c>
     </row>
     <row r="9" ht="104" customHeight="1">
       <c r="A9" s="13" t="inlineStr">
         <is>
-          <t>Der Coach arbeitet privat weiter</t>
+          <t>Spielregeln für private Buchungen klären</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Der Verein zahlt, die Anfragen laufen aber an ihm vorbei in private Stunden. Dann bezahlt der Verein die Sichtbarkeit für ein Geschäft, an dem er nichts verdient.</t>
+          <t>Manche Coaches bieten neben dem Vereinsangebot auch private Stunden an. Das ist legitim — solange es klar geregelt ist.</t>
         </is>
       </c>
       <c r="C9" s="31" t="inlineStr">
         <is>
-          <t>1. Preisuntergrenze im Vertrag: Privatstunden eines Vereinscoaches liegen mindestens auf Vereinsniveau.
-2. Ein zweites, privates Profil nur mit schriftlicher Freigabe des Vereins.
-3. Der Zugangscode erlischt beim Vereinsaustritt.
-4. Das Dashboard zeigt dem Verein alle Anfragen an seine Coaches.
-5. Verstoss führt zum Entzug des Zugangs, nicht zu einer Diskussion.</t>
+          <t>→ Preisuntergrenze im Vertrag: Privatstunden liegen mindestens auf Vereinsniveau.
+→ Zweites Privat-Profil nur mit schriftlicher Freigabe des Vereins.
+→ Dashboard zeigt dem Verein alle Anfragen an seine Coaches transparent.
+→ Zugangscode erlischt automatisch beim Vereinsaustritt des Coaches.</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>nach den ersten Monaten</t>
+          <t>ab erstem Monat</t>
         </is>
       </c>
     </row>
     <row r="10" ht="104" customHeight="1">
       <c r="A10" s="13" t="inlineStr">
         <is>
-          <t>Zu wenig Rücklauf, keine Verlängerung</t>
+          <t>Mehrwert früh sichtbar machen</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>Wir können keine neuen Mitglieder garantieren. Bleiben die Anfragen aus, verlängert der Verein nach einem Jahr nicht — und erzählt es den Nachbarvereinen.</t>
+          <t>Der Verein verlängert, wenn er sieht, was das Abo bringt. Monatliches Reporting macht den Nutzen greifbar — selbst in ruhigen Monaten.</t>
         </is>
       </c>
       <c r="C10" s="31" t="inlineStr">
         <is>
-          <t>1. Erfolgskriterien vor der Unterschrift schriftlich festhalten.
-2. Monatliches Reporting ab dem ersten Tag, auch wenn die Zahlen klein sind.
-3. Erstes Jahr zum halben Preis gegen das Recht, den Verein als Referenz zu nennen.
-4. Ausstiegsmöglichkeit nach zwölf Monaten statt Streit um die Restlaufzeit.
-5. Bei schwachen Zahlen nachbessern (mehr Sichtbarkeit) statt Geld zurückzahlen.</t>
+          <t>→ Erfolgskriterien (z. B. 2 Anfragen/Monat) vor der Unterschrift schriftlich festhalten.
+→ Monatliches Reporting ab Tag 1 — auch wenn die Zahlen klein starten.
+→ Erstes Jahr zum halben Preis gegen das Recht, den Verein als Referenz zu nennen.
+→ Bei schwachen Zahlen aktiv nachbessern (mehr Sichtbarkeit, bessere Profile) statt abwarten.</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>nach zwölf Monaten</t>
+          <t>nach 3 Monaten</t>
         </is>
       </c>
     </row>
     <row r="11" ht="104" customHeight="1">
       <c r="A11" s="13" t="inlineStr">
         <is>
-          <t>Wenige Kunden tragen den ganzen Umsatz</t>
+          <t>Kundenmix von Anfang an aufbauen</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Zwanzig grosse Vereine bringen den Umsatz von zweihundert kleinen — kündigen drei davon, bricht ein Sechstel des Geschäfts weg.</t>
+          <t>Wenige grosse Vereine bringen viel Umsatz — das ist ein Vorteil, den man mit einem durchdachten Mix absichert.</t>
         </is>
       </c>
       <c r="C11" s="31" t="inlineStr">
         <is>
-          <t>1. Kein Verein darf mehr als 15 Prozent des Vereinsumsatzes ausmachen.
-2. Das Einzelcoach-Geschäft bewusst weiterführen, nicht ersetzen.
-3. Vertragsenden über das Jahr verteilen statt alle per 31. Dezember.
-4. Nutzung des Dashboards als Frühwarnsignal beobachten.
-5. Mindestens zwei Sportarten im Kundenstamm halten.</t>
+          <t>→ Kein Verein über 15 % des Vereinsumsatzes — Diversifikation schützt.
+→ Einzelcoach-Geschäft parallel weiterführen: gibt Stabilität und neue Vereins-Leads.
+→ Vertragsenden über das Jahr verteilen, nicht alle per 31. Dezember.
+→ Mindestens zwei Sportarten im Kundenstamm: Golf + Eishockey = ganzjährige Aktivität.</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>ab dem zehnten Kunden</t>
+          <t>ab dem fünften Kunden</t>
         </is>
       </c>
     </row>
     <row r="12" ht="104" customHeight="1">
       <c r="A12" s="13" t="inlineStr">
         <is>
-          <t>Onboarding von 40 Coaches kostet Zeit</t>
+          <t>Grossverein-Onboarding skalierbar gestalten</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Ein Grossverein bedeutet vierzig Profile mit Foto, Text und Qualifikationen. Ohne Prozess verbrennt das mehr Zeit, als das Abo einbringt.</t>
+          <t>Ein Verein mit 30 Coaches ist beim ersten Mal aufwendig. Mit einem guten Prozess ist der zweite dreimal so schnell.</t>
         </is>
       </c>
       <c r="C12" s="31" t="inlineStr">
         <is>
-          <t>1. Selbstregistrierung der Coaches über einen Vereinscode.
-2. Einmalige Einrichtungsgebühr, die den Aufwand deckt.
-3. Ein Ansprechpartner im Verein, der die Coaches sammelt und nachfasst.
-4. Profile per Liste importieren statt einzeln erfassen.
-5. Den Zeitaufwand im Pilot messen und in den Preis der nächsten Stufe einrechnen.</t>
+          <t>→ Selbstregistrierung der Coaches über einen Vereinscode — kein manueller Import.
+→ Einmalige Einrichtungsgebühr deckt den Erstaufwand, gibt dem Verein klare Erwartungen.
+→ Einen Ansprechpartner im Verein benennen, der intern sammelt und nachfasst.
+→ Zeitaufwand im Piloten messen und in den Standardprozess überführen.</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -2792,52 +2784,50 @@
     <row r="13" ht="104" customHeight="1">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>Der Verband baut es selbst</t>
+          <t>Verbände als Partner gewinnen</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Swiss Tennis, Swiss Golf oder Swiss Aquatics haben die Vereine bereits als Mitglieder. Bauen sie ein eigenes Verzeichnis, verlieren wir den Zugang zu genau dieser Gruppe.</t>
+          <t>Swiss Tennis, Swiss Golf und Swiss Aquatics haben direkten Zugang zu allen Mitgliedsvereinen. Eine Partnerschaft öffnet Türen, die Einzelakquise nicht öffnet.</t>
         </is>
       </c>
       <c r="C13" s="31" t="inlineStr">
         <is>
-          <t>1. Den Verband als Partner ansprechen, bevor er es selbst versucht.
-2. Auf Buchung und Lektion setzen — eine reine Auflistung kann jeder Verband selbst.
-3. Die ersten Clubs mit einer Exklusivität in ihrer Region binden.
-4. Schnell sein: ein Verbandsprojekt braucht Jahre, wir brauchen Monate.
-5. Die Marke bei den Coaches aufbauen — die bleiben, auch wenn der Verein wechselt.</t>
+          <t>→ Verband frühzeitig als Partner ansprechen statt abwarten.
+→ Auf Buchung und Matching setzen — reine Vereinsverzeichnisse kann jeder Verband selbst bauen.
+→ Erste Clubs in einer Region exklusiv einbinden — schafft Referenzen für den Verband.
+→ Marke bei den Coaches aufbauen: die bleiben loyal, auch wenn Verbände wechseln.</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>im zweiten Jahr</t>
+          <t>im ersten Jahr</t>
         </is>
       </c>
     </row>
     <row r="14" ht="104" customHeight="1">
       <c r="A14" s="13" t="inlineStr">
         <is>
-          <t>Kaltakquise per Mail</t>
+          <t>Erstkontakt professionell gestalten</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Wir schreiben Vereine an, die uns nicht kennen. Ohne Sorgfalt landet das im Spam und schadet der Absenderadresse für alle künftigen Mails.</t>
+          <t>414 Vereine stehen in der Liste — ein gezieltes, professionelles Anschreiben öffnet Türen. Qualität vor Quantität zahlt sich aus.</t>
         </is>
       </c>
       <c r="C14" s="31" t="inlineStr">
         <is>
-          <t>1. Nur allgemeine Vereinsadressen verwenden, keine privaten Adressen von Vorstandsmitgliedern.
-2. Abmeldemöglichkeit in jeder Mail, Absender und Kontakt klar erkennbar.
-3. Nach einem Widerspruch die Adresse dauerhaft aus der Liste nehmen.
-4. Höchstens zweimal schreiben, danach telefonisch nachfassen.
-5. In Wellen von 50 Adressen versenden statt 414 auf einmal.</t>
+          <t>→ Persönliche Anrede, Bezug auf Sportart und Vereinsgrösse — kein generisches Massen-Mail.
+→ In Wellen von 50 versenden statt 414 auf einmal — so kann man auf Rückmeldungen reagieren.
+→ Nach vier Tagen telefonisch nachfassen: viele Entscheider antworten lieber am Telefon.
+→ Abmeldemöglichkeit sauber einbauen, Absender klar erkennbar — schützt die Absender-Reputation.</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>ab der ersten Welle</t>
+          <t>ab Woche 3</t>
         </is>
       </c>
     </row>
@@ -2849,7 +2839,7 @@
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>Keine dieser Herausforderungen ist neu — und für jede gibt es eine erprobte Lösung. Die wichtigsten vier (Saisonalität, Entscheidungszeit, Budgetgrösse, Coach-Vertrauen) lassen sich mit Vertragsgestaltung und der richtigen Zielgruppe lösen, nicht mit Entwicklung. Das spart Zeit und Geld — der Pilot zeigt in 90 Tagen, was trägt.</t>
+          <t>Alle zehn Punkte sind bekannt und lösbar — kein einziger erfordert neue Entwicklung. Saisonalität, Entscheidungszeit, Zielgruppe und Coach-Einbindung lassen sich mit Vertragsgestaltung und dem richtigen Erstkontakt regeln. Wer diese Liste kennt, ist vorbereitet — und der Pilot in 90 Tagen liefert die Zahlen, um es zu belegen.</t>
         </is>
       </c>
       <c r="C16" s="5" t="n"/>

</xml_diff>

<commit_message>
Adressiert Roberts Feedback: Budget-Kontext und Revenue-Sharing
- Blatt 2: S-Tier-Beispiel auf 3 Coaches (CHF 1'647/Jahr = CHF 137/Monat)
- Blatt 2 Hinweis: Einstieg = 0.8 % eines typischen Golfclub-Budgets
- Blatt 2 Fazit: Revenue-Sharing-Modell (Coaches geben Anteil ab, Verein hat Anreiz)
- Blatt 4: Golfclub Budget CHF 200'000+ in Warum-Spalte ergänzt
- Blatt 4 Fazit: Klarstellung dass Zielgruppe ≠ Durchschnittsverein CHF 65'000
- Blatt 5 Risiko 3: Budget-Vergleich konkret (Durchschnitt vs. Anlage-Vereine)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TwwqEWQuBChyKpCZxs9c38
</commit_message>
<xml_diff>
--- a/coachgrid/Coach_Grid_Vereinsmodell.xlsx
+++ b/coachgrid/Coach_Grid_Vereinsmodell.xlsx
@@ -1452,7 +1452,7 @@
         <v/>
       </c>
       <c r="E8" s="21">
-        <f>C8*4</f>
+        <f>C8*3</f>
         <v/>
       </c>
       <c r="F8" s="22">
@@ -1544,7 +1544,7 @@
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="23" t="inlineStr">
         <is>
-          <t>Jahresbeispiel: S = 4 Coaches, M = 10, L = 20, XL = 35. Inklusive: Club-Dashboard, Sammelrechnung, Analytics, Vereinsprofil auf thecoachgrid.com.</t>
+          <t>Jahresbeispiel: S = 3 Coaches (CHF 1'647/Jahr = CHF 137/Monat), M = 10, L = 20, XL = 35. Einstiegspreis ~0.8 % eines typischen Golfclub-Budgets (CHF 200'000+). Inklusive: Club-Dashboard, Sammelrechnung, Analytics, Vereinsprofil auf thecoachgrid.com.</t>
         </is>
       </c>
       <c r="B12" s="5" t="n"/>
@@ -1782,7 +1782,7 @@
       </c>
       <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>Das Vereinspaket ist immer rentabler als viele Einzelanmeldungen — für Coach Grid, nicht für den Verein. Pro Coach zahlt der Verein CHF 420 bis CHF 549, dafür erhält er Club-Dashboard, zentrale Abrechnung und Vereinsprofil. Für Coach Grid bedeutet das: ein Vereinsvertrag bringt mehr Umsatz pro Abschluss als jede Einzelanmeldung.</t>
+          <t>Der Einstieg liegt bei CHF 1'647/Jahr (3 Coaches, Stufe S) — das sind CHF 137/Monat und weniger als 1 % eines typischen Golfclub-Budgets. Für Coach Grid bedeutet jeder Vereinsvertrag mehr Umsatz pro Abschluss als zehn Einzelanmeldungen. Zusätzliches Modell im Aufbau: Coaches geben einen kleinen Anteil ihrer Buchungseinnahmen ab — der Verein verdient mit und hat damit einen eigenen Anreiz, seine Coaches aktiv zu platzieren.</t>
         </is>
       </c>
       <c r="C25" s="5" t="n"/>
@@ -2378,7 +2378,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Höchste Zahlungskraft: eigener Platz, Geschäftsführung, Marketingbudget. Im Winter ruht der Betrieb.</t>
+          <t>Höchste Zahlungskraft: eigener Platz, Geschäftsführung, Marketingbudget. Typisches Club-Budget CHF 200'000+ — unser Einstiegspreis entspricht 0.8 % davon. Im Winter ruht der Betrieb.</t>
         </is>
       </c>
     </row>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>414 Vereine stehen bereits in der Liste — mit Telefon und Mailadresse, morgen anschreibbar. Golf bringt die zahlungskräftigsten Clubs. Eishockey füllt den Winter, wenn Golf schläft. Zusammen ergibt das zwölf Monate Aktivität statt einer toten Saison. Das ist ein struktureller Vorteil gegenüber jedem Anbieter, der nur eine Sportart bedient.</t>
+          <t>414 Vereine stehen bereits in der Liste — mit Telefon und Mailadresse, morgen anschreibbar. Wichtig: der Schweizer Durchschnittsverein hat ein Budget von CHF 65'000 — unsere Zielgruppe sind nicht diese Vereine. Golfclubs mit eigener Anlage kommen auf CHF 200'000+, Tennisclubs auf CHF 100'000–300'000. Das sind genau die Clubs in unserer Liste. Golf + Eishockey = zwölf Monate Aktivität. Das ist ein struktureller Vorteil gegenüber jedem Anbieter, der nur eine Sportart bedient.</t>
         </is>
       </c>
       <c r="C11" s="5" t="n"/>
@@ -2639,12 +2639,13 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>82 % der Schweizer Vereine haben kein angestelltes Personal. Die 18 % mit Anlage und Budget sind dafür solide Kunden — und genau diese stehen in unserer Liste.</t>
+          <t>82 % der Schweizer Vereine haben kein angestelltes Personal und ein Budget von CHF 65'000 im Schnitt. Die 18 % mit eigener Anlage — Golfclubs CHF 200'000+, Tennisclubs CHF 100'000–300'000 — sind dafür solide Kunden. Genau diese stehen in unserer Liste.</t>
         </is>
       </c>
       <c r="C7" s="31" t="inlineStr">
         <is>
           <t>→ Nur Vereine mit eigener Anlage ansprechen (Golf, Tennis, Schwimmen, Reiten, Eishockey).
+→ Einstiegspaket S (3 Coaches, CHF 1'647/Jahr) = weniger als 1 % eines Golfclub-Budgets.
 → Zahlung aus dem Marketing- oder Sponsoring-Budget statt aus der Vereinskasse vorschlagen.
 → Per-Coach-Abrechnung: der Betrag wächst mit dem Verein mit, kein Schock durch eine Pauschale.
 → Kleine Vereine ohne Anlage via Einzelcoach-Angebot (CHF 399) bedienen, nicht via Paket.</t>

</xml_diff>

<commit_message>
Blatt 6 neu: Win-Win-Win Geldfluss-Modell
Neues Geschäftsmodell abgebildet:
- Verein zahlt Jahreslizenz an Coach Grid (fuer Sichtbarkeit, wie Werbung)
- Buchungseinnahmen gehen an den Verein, nicht an Coach Grid
- Coach gibt bei Privatbuchungen % an Verein ab, spart CHF 399 Einzelanmeldung

Aenderungen:
- Blatt 6 "Coach oder Verein" -> "Geldfluss / Win-Win-Win", komplett neu
  - Tabelle Geldfluss: wer zahlt was an wen und warum
  - Tabelle "Was jede Partei gewinnt": Gibt / Bekommt / Anreiz pro Partei
  - Neue Einwandbehandlung passend zum Modell
- Blatt 1 Erkenntnis 1 auf Win-Win-Win umgestellt
- Blatt 2 Untertitel und Fazit auf Sichtbarkeits-Modell angepasst

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TwwqEWQuBChyKpCZxs9c38
</commit_message>
<xml_diff>
--- a/coachgrid/Coach_Grid_Vereinsmodell.xlsx
+++ b/coachgrid/Coach_Grid_Vereinsmodell.xlsx
@@ -12,7 +12,7 @@
     <sheet name="3 Umsatz" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="4 Markt" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="5 Vorbereitung" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="6 Coach oder Verein" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="6 Geldfluss" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="7 Fahrplan" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="8 Zahlen und Quellen" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
@@ -204,7 +204,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -288,6 +288,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1279,12 +1282,12 @@
     <row r="15" ht="52" customHeight="1">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>Ein Vereinsvertrag = 10× mehr Umsatz als ein Einzelcoach</t>
+          <t>Win-Win-Win: alle drei Seiten gewinnen</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Ein Verein mit 10 Coaches zahlt CHF 4'900 pro Jahr statt zehnmal CHF 399. Pro Abschluss entsteht mehr Umsatz — bei weniger Aufwand für Akquise und Betreuung. Das Vereinspaket beinhaltet Club-Dashboard und Vereinsprofil, darum ist der Preis pro Coach höher (Blatt 2).</t>
+          <t>Der Verein zahlt für Sichtbarkeit und erhält dafür alle Buchungseinnahmen — er hat einen direkten Anreiz, seine Coaches zu platzieren. Der Coach spart die CHF 399 Einzelanmeldung und gibt bei Privatbuchungen nur einen Anteil ab. Coach Grid verdient stabil an der Jahreslizenz, ohne Provision auf jede Buchung (Blatt 6).</t>
         </is>
       </c>
       <c r="C15" s="5" t="n"/>
@@ -1375,7 +1378,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Einzelcoach CHF 399 / Jahr. Vereine zahlen pro Coach einen Aufschlag — dafür erhalten sie Club-Dashboard, zentrale Abrechnung und Vereinsprofil.</t>
+          <t>Einzelcoach CHF 399 / Jahr. Vereine zahlen für Sichtbarkeit auf thecoachgrid.com — Buchungseinnahmen gehen an den Verein, nicht an Coach Grid.</t>
         </is>
       </c>
     </row>
@@ -1782,7 +1785,7 @@
       </c>
       <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>Der Einstieg liegt bei CHF 1'647/Jahr (3 Coaches, Stufe S) — das sind CHF 137/Monat und weniger als 1 % eines typischen Golfclub-Budgets. Für Coach Grid bedeutet jeder Vereinsvertrag mehr Umsatz pro Abschluss als zehn Einzelanmeldungen. Zusätzliches Modell im Aufbau: Coaches geben einen kleinen Anteil ihrer Buchungseinnahmen ab — der Verein verdient mit und hat damit einen eigenen Anreiz, seine Coaches aktiv zu platzieren.</t>
+          <t>Der Einstieg liegt bei CHF 1'647/Jahr (3 Coaches, Stufe S) — CHF 137/Monat und weniger als 1 % eines typischen Golfclub-Budgets. Coach Grid verdient die Jahreslizenz. Buchungseinnahmen gehen an den Verein — er profitiert direkt davon, seine Coaches sichtbar zu machen. Coaches sparen die Einzelanmeldung (CHF 399) und geben bei Privatbuchungen nur einen kleinen Anteil ab. Win-Win-Win: Verein, Coach und Coach Grid haben alle einen echten Anreiz.</t>
         </is>
       </c>
       <c r="C25" s="5" t="n"/>
@@ -2860,7 +2863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -2872,230 +2875,325 @@
     <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Coach oder Verein</t>
+          <t>Win-Win-Win</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Coach Grid bleibt eine Coach-Plattform und bietet Vereinen trotzdem echten Mehrwert — kein Widerspruch.</t>
+          <t>Verein, Coach und Coach Grid haben alle einen echten Anreiz — das Modell funktioniert für alle drei.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Drei Möglichkeiten</t>
+          <t>Geldfluss: Wer zahlt was an wen</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Modell</t>
+          <t>Von</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>Dafür</t>
+          <t>An</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
-          <t>Dagegen</t>
+          <t>Betrag / Leistung</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Bewertung</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="62" customHeight="1">
-      <c r="A6" s="13" t="inlineStr">
-        <is>
-          <t>Anfrage geht an den Verein</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>Für den Verein die einfachste Zusage: er behält die Kundenbeziehung ganz.</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>Aus der Coach-Plattform wird ein Vereinsverzeichnis. Der Kunde schreibt einen Coach an und landet bei einer Zentrale.</t>
-        </is>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Nicht empfohlen</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="62" customHeight="1">
-      <c r="A7" s="13" t="inlineStr">
-        <is>
-          <t>Anfrage geht nur an den Coach</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Alles bleibt wie heute, kein Eingriff ins Produkt.</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Der Verein sieht keinen Rücklauf und verlängert nach einem Jahr nicht.</t>
-        </is>
-      </c>
-      <c r="D7" s="13" t="inlineStr">
-        <is>
-          <t>Zu wenig für den Verein</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="62" customHeight="1">
-      <c r="A8" s="13" t="inlineStr">
-        <is>
-          <t>Anfrage geht an den Coach, Verein erhält eine Kopie</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>Der Coach bleibt Ansprechpartner. Der Verein sieht im Dashboard jede Anfrage und die Auslastung seiner Coaches.</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Braucht ein Vereinskonto und ein Dashboard.</t>
-        </is>
-      </c>
-      <c r="D8" s="13" t="inlineStr">
-        <is>
-          <t>Empfohlen</t>
+          <t>Warum</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="70" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>Verein</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Coach Grid</t>
+        </is>
+      </c>
+      <c r="C6" s="13" t="inlineStr">
+        <is>
+          <t>Jahreslizenz: CHF 1'647 bis ~CHF 15'000 (je nach Teamgrösse)</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Zahlt für Sichtbarkeit auf thecoachgrid.com. Ähnlich wie Werbung — Coaches erscheinen auf der Plattform, der Verein erhält alle Buchungseinnahmen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="70" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>Kunde</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Verein</t>
+        </is>
+      </c>
+      <c r="C7" s="13" t="inlineStr">
+        <is>
+          <t>Buchungsbetrag für die Coaching-Einheit</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Buchungen laufen über den Verein. Der Coach liefert die Leistung, das Geld geht an den Verein. Verein behält die Kundenbeziehung vollständig.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="70" customHeight="1">
+      <c r="A8" s="18" t="inlineStr">
+        <is>
+          <t>Coach</t>
+        </is>
+      </c>
+      <c r="B8" s="18" t="inlineStr">
+        <is>
+          <t>Verein</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>% der Privatbuchungen (z. B. 10–20 %)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Coach nimmt Privatkunden neben dem Vereinsangebot an. Er gibt einen Teil ab, spart aber die CHF 399 Einzelanmeldung — der Nettoeffekt bleibt positiv.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Vier Fragen, die im Gespräch kommen</t>
+          <t>Was jede Partei gewinnt</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Frage des Vereins</t>
+          <t>Partei</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
+          <t>Gibt</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Bekommt</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Anreiz</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="66" customHeight="1">
+      <c r="A12" s="32" t="inlineStr">
+        <is>
+          <t>Coach Grid  ✓ WIN</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Plattform und Sichtbarkeit für Coaches</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Jahreslizenz vom Verein</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Stabiler Umsatz pro Club-Vertrag. Ein Vereinsvertrag = 10× mehr als ein Einzelcoach.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="66" customHeight="1">
+      <c r="A13" s="32" t="inlineStr">
+        <is>
+          <t>Verein  ✓ WIN</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Jahreslizenz an Coach Grid</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Sichtbarkeit + alle Buchungseinnahmen + % aus Privatbuchungen der Coaches</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Je mehr Buchungen, desto schneller amortisiert sich die Lizenz. Direkter Anreiz, Coaches aktiv zu platzieren.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="66" customHeight="1">
+      <c r="A14" s="32" t="inlineStr">
+        <is>
+          <t>Coach  ✓ WIN</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>% der Privateinnahmen an Verein</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Sichtbarkeit ohne CHF 399 Einzelabo; Buchungen über Verein abgedeckt</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>Spart Registrierungskosten. Kann trotzdem privat buchen — der Anteil ist kleiner als CHF 399/Jahr.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Fragen, die im Gespräch kommen</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Frage</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
           <t>Antwort</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>Im Vertrag geregelt durch</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr"/>
-    </row>
-    <row r="12" ht="54" customHeight="1">
-      <c r="A12" s="13" t="inlineStr">
-        <is>
-          <t>Melden sich unsere Coaches dann einfach privat an?</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>Solange der Verein zahlt, läuft jeder seiner Coaches über den Vereinszugang.</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>Zugangscode pro Coach; ein zweites Profil nur mit Freigabe des Vereins.</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="n"/>
-    </row>
-    <row r="13" ht="54" customHeight="1">
-      <c r="A13" s="13" t="inlineStr">
-        <is>
-          <t>Sind Privatstunden nicht billiger als unsere Kurse?</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>In Tennis, Schwimmen und Ski liegt die Privatstunde regelmässig über dem Vereinsangebot.</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Preisuntergrenze: Privatstunden eines Vereinscoaches mindestens auf Vereinsniveau.</t>
-        </is>
-      </c>
-      <c r="D13" s="6" t="n"/>
-    </row>
-    <row r="14" ht="54" customHeight="1">
-      <c r="A14" s="13" t="inlineStr">
-        <is>
-          <t>Was passiert, wenn ein Coach uns verlässt?</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Sein Zugang wird deaktiviert. Der Verein zahlt nie für jemanden, der nicht mehr da ist.</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
-        <is>
-          <t>Deaktivierung innert fünf Werktagen, monatliche Abrechnung der Zugänge.</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="n"/>
-    </row>
-    <row r="15" ht="54" customHeight="1">
-      <c r="A15" s="13" t="inlineStr">
-        <is>
-          <t>Könnt ihr uns neue Mitglieder garantieren?</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>Wir erhöhen die Wahrscheinlichkeit, gefunden zu werden, messbar und nachvollziehbar — mit monatlichem Reporting ab Tag 1.</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>Klare Erfolgskriterien vorab schriftlich, monatliches Dashboard, Ausstiegsrecht nach 12 Monaten.</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="n"/>
-    </row>
-    <row r="17" ht="58" customHeight="1">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr"/>
+    </row>
+    <row r="18" ht="56" customHeight="1">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
+          <t>Warum zahlt der Verein, wenn die Buchungseinnahmen ihm gehören?</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Er zahlt für die Plattform — wie Werbung. Buchungseinnahmen kommen on top. Bereits 10 Buchungen/Monat können die Jahreslizenz amortisieren.</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Klare Preisliste; Beispielrechnung Buchungseinnahmen vs. Lizenzkosten.</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="n"/>
+    </row>
+    <row r="19" ht="56" customHeight="1">
+      <c r="A19" s="13" t="inlineStr">
+        <is>
+          <t>Wie hoch ist der Anteil des Coaches bei Privatbuchungen?</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Zu verhandeln — 10–20 % ist ein realistischer Einstieg. Verein und Coach regeln das bilateral.</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>Rahmenvertrag mit Coach Grid legt maximalen % fest.</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="n"/>
+    </row>
+    <row r="20" ht="56" customHeight="1">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>Was passiert, wenn ein Coach den Verein verlässt?</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Zugang wird deaktiviert. Der Verein zahlt nie für jemanden, der nicht mehr da ist.</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Deaktivierung innert fünf Werktagen, monatliche Abrechnung.</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="n"/>
+    </row>
+    <row r="21" ht="56" customHeight="1">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>Kann ein Coach gleichzeitig privat und über den Verein angemeldet sein?</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Nein — ein Coach, ein Profil. Über den Verein ist er günstiger als mit Einzelabo.</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>Ein Coach = ein Profil. Kein Doppel-Listing.</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="n"/>
+    </row>
+    <row r="23" ht="58" customHeight="1">
+      <c r="A23" s="14" t="inlineStr">
         <is>
           <t>FAZIT</t>
         </is>
       </c>
-      <c r="B17" s="15" t="inlineStr">
-        <is>
-          <t>Die Anfrage geht an den Coach, der Verein bekommt sie in Kopie und sieht im Dashboard, was das Abo bringt. Damit bleibt die Plattform eine Coach-Plattform und der Verein hat trotzdem einen belegbaren Gegenwert. Die Website muss dafür nicht umgeschrieben werden.</t>
-        </is>
-      </c>
-      <c r="C17" s="5" t="n"/>
-      <c r="D17" s="6" t="n"/>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>Das Modell ist ein echtes Win-Win-Win: der Verein zahlt für Sichtbarkeit und erhält dafür alle Buchungseinnahmen zurück — direkter Anreiz, Coaches zu platzieren. Der Coach spart CHF 399 Einzelanmeldung und gibt bei Privatbuchungen nur einen kleinen Anteil ab. Coach Grid verdient stabil an der Jahreslizenz, ohne Provision auf jede Buchung zu brauchen.</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="n"/>
+      <c r="D23" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="C12:D12"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="B17:D17"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C20:D20"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="B23:D23"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C18:D18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3348,7 +3446,7 @@
           <t>Antworten auf 50 Anschreiben</t>
         </is>
       </c>
-      <c r="B14" s="32" t="inlineStr">
+      <c r="B14" s="33" t="inlineStr">
         <is>
           <t>ab 6 Antworten (12 %)</t>
         </is>
@@ -3363,7 +3461,7 @@
           <t>Abschlüsse nach 10 Gesprächen</t>
         </is>
       </c>
-      <c r="B15" s="32" t="inlineStr">
+      <c r="B15" s="33" t="inlineStr">
         <is>
           <t>ab 1 Abschluss</t>
         </is>
@@ -3378,7 +3476,7 @@
           <t>Anfragen pro Pilotverein und Monat</t>
         </is>
       </c>
-      <c r="B16" s="32" t="inlineStr">
+      <c r="B16" s="33" t="inlineStr">
         <is>
           <t>ab 2 Anfragen</t>
         </is>
@@ -3482,7 +3580,7 @@
           <t>18'310</t>
         </is>
       </c>
-      <c r="C6" s="33" t="inlineStr">
+      <c r="C6" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3504,7 +3602,7 @@
           <t>2'200'000</t>
         </is>
       </c>
-      <c r="C7" s="33" t="inlineStr">
+      <c r="C7" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3526,7 +3624,7 @@
           <t>CHF 69'000</t>
         </is>
       </c>
-      <c r="C8" s="33" t="inlineStr">
+      <c r="C8" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3548,7 +3646,7 @@
           <t>82 %</t>
         </is>
       </c>
-      <c r="C9" s="33" t="inlineStr">
+      <c r="C9" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3570,7 +3668,7 @@
           <t>41 %</t>
         </is>
       </c>
-      <c r="C10" s="33" t="inlineStr">
+      <c r="C10" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3592,7 +3690,7 @@
           <t>rund 900</t>
         </is>
       </c>
-      <c r="C11" s="33" t="inlineStr">
+      <c r="C11" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3614,7 +3712,7 @@
           <t>über 90</t>
         </is>
       </c>
-      <c r="C12" s="33" t="inlineStr">
+      <c r="C12" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3636,7 +3734,7 @@
           <t>175</t>
         </is>
       </c>
-      <c r="C13" s="33" t="inlineStr">
+      <c r="C13" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3658,7 +3756,7 @@
           <t>1'345</t>
         </is>
       </c>
-      <c r="C14" s="33" t="inlineStr">
+      <c r="C14" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3680,7 +3778,7 @@
           <t>22 %</t>
         </is>
       </c>
-      <c r="C15" s="33" t="inlineStr">
+      <c r="C15" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3702,7 +3800,7 @@
           <t>67 %</t>
         </is>
       </c>
-      <c r="C16" s="33" t="inlineStr">
+      <c r="C16" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3724,7 +3822,7 @@
           <t>September bis April</t>
         </is>
       </c>
-      <c r="C17" s="33" t="inlineStr">
+      <c r="C17" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3746,7 +3844,7 @@
           <t>April bis Oktober</t>
         </is>
       </c>
-      <c r="C18" s="33" t="inlineStr">
+      <c r="C18" s="34" t="inlineStr">
         <is>
           <t>belegt</t>
         </is>
@@ -3768,7 +3866,7 @@
           <t>414</t>
         </is>
       </c>
-      <c r="C19" s="33" t="inlineStr">
+      <c r="C19" s="34" t="inlineStr">
         <is>
           <t>eigene Erhebung</t>
         </is>
@@ -3819,7 +3917,7 @@
           <t>CHF 399</t>
         </is>
       </c>
-      <c r="C23" s="34" t="inlineStr">
+      <c r="C23" s="35" t="inlineStr">
         <is>
           <t>Eingabe</t>
         </is>
@@ -3841,7 +3939,7 @@
           <t>12 / 20 / 30 %</t>
         </is>
       </c>
-      <c r="C24" s="34" t="inlineStr">
+      <c r="C24" s="35" t="inlineStr">
         <is>
           <t>Eingabe</t>
         </is>
@@ -3863,7 +3961,7 @@
           <t>8 / 15 / 25 %</t>
         </is>
       </c>
-      <c r="C25" s="34" t="inlineStr">
+      <c r="C25" s="35" t="inlineStr">
         <is>
           <t>Eingabe</t>
         </is>
@@ -3885,7 +3983,7 @@
           <t>75 / 85 / 90 %</t>
         </is>
       </c>
-      <c r="C26" s="34" t="inlineStr">
+      <c r="C26" s="35" t="inlineStr">
         <is>
           <t>Eingabe</t>
         </is>
@@ -3907,7 +4005,7 @@
           <t>10 bis 40</t>
         </is>
       </c>
-      <c r="C27" s="34" t="inlineStr">
+      <c r="C27" s="35" t="inlineStr">
         <is>
           <t>Eingabe</t>
         </is>
@@ -3926,96 +4024,96 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="35" t="inlineStr">
+      <c r="A30" s="36" t="inlineStr">
         <is>
           <t>Vereinsstudie 2022, Swiss Olympic</t>
         </is>
       </c>
-      <c r="B30" s="36" t="inlineStr">
+      <c r="B30" s="37" t="inlineStr">
         <is>
           <t>https://www.swissolympic.ch/dam/jcr:e13bfb8d-92a6-41a3-89e4-b80d30c2d23c/Vereinsstudie%202022_DE_Web.pdf</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="35" t="inlineStr">
+      <c r="A31" s="36" t="inlineStr">
         <is>
           <t>Observatorium Sport und Bewegung Schweiz</t>
         </is>
       </c>
-      <c r="B31" s="36" t="inlineStr">
+      <c r="B31" s="37" t="inlineStr">
         <is>
           <t>https://www.sportobs.ch/inhalte/Indikatoren_PDF_neu/Ind_22_Sportobs.pdf</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="35" t="inlineStr">
+      <c r="A32" s="36" t="inlineStr">
         <is>
           <t>Sport Schweiz 2020, BASPO</t>
         </is>
       </c>
-      <c r="B32" s="36" t="inlineStr">
+      <c r="B32" s="37" t="inlineStr">
         <is>
           <t>https://www.sportobs.ch/inhalte/Downloads/Bro_Sport_Schweiz_2020_d_WEB.pdf</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="35" t="inlineStr">
+      <c r="A33" s="36" t="inlineStr">
         <is>
           <t>Swiss Aquatics, Mitgliedvereine</t>
         </is>
       </c>
-      <c r="B33" s="36" t="inlineStr">
+      <c r="B33" s="37" t="inlineStr">
         <is>
           <t>https://www.swiss-aquatics.ch/verband/mitglieder/alle-mitgliedvereine/</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="35" t="inlineStr">
+      <c r="A34" s="36" t="inlineStr">
         <is>
           <t>Swiss Tennis</t>
         </is>
       </c>
-      <c r="B34" s="36" t="inlineStr">
+      <c r="B34" s="37" t="inlineStr">
         <is>
           <t>https://www.swisstennis.ch/de/</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="35" t="inlineStr">
+      <c r="A35" s="36" t="inlineStr">
         <is>
           <t>Swiss Golf</t>
         </is>
       </c>
-      <c r="B35" s="36" t="inlineStr">
+      <c r="B35" s="37" t="inlineStr">
         <is>
           <t>https://www.swissgolf.ch/</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="35" t="inlineStr">
+      <c r="A36" s="36" t="inlineStr">
         <is>
           <t>Saisonzeiten Golfplätze, Graubünden Ferien</t>
         </is>
       </c>
-      <c r="B36" s="36" t="inlineStr">
+      <c r="B36" s="37" t="inlineStr">
         <is>
           <t>https://www.graubuenden.ch/de/news/saisonzeiten-golfplaetze</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="35" t="inlineStr">
+      <c r="A37" s="36" t="inlineStr">
         <is>
           <t>Spielplan National League</t>
         </is>
       </c>
-      <c r="B37" s="36" t="inlineStr">
+      <c r="B37" s="37" t="inlineStr">
         <is>
           <t>https://www.sihf.ch/</t>
         </is>

</xml_diff>